<commit_message>
* Bringing in static files from main
</commit_message>
<xml_diff>
--- a/app/static/returns/returns.xlsx
+++ b/app/static/returns/returns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work Files\ips generator\ips_generator\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8FFEC3-FEEF-4121-9693-7772F8BE33C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3799630-C69A-4CBE-A1E3-585352F4DA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8205" yWindow="3975" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
+    <workbookView xWindow="3555" yWindow="4800" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -780,52 +780,52 @@
         <v>25</v>
       </c>
       <c r="C2" s="2">
-        <v>1.24508333333333E-2</v>
+        <v>-5.1765416666667008E-3</v>
       </c>
       <c r="D2" s="2">
-        <v>1.6722055828822361E-2</v>
+        <v>2.7077582276642479E-2</v>
       </c>
       <c r="E2" s="2">
-        <v>3.2421957557520642E-2</v>
+        <v>2.7077582276642479E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>0.1049618127567562</v>
+        <v>8.760456306811637E-2</v>
       </c>
       <c r="G2" s="2">
-        <v>3.8563021682313181E-2</v>
+        <v>3.9439975710667152E-2</v>
       </c>
       <c r="H2" s="2">
-        <v>6.1502983721945848E-2</v>
+        <v>6.3877404467325816E-2</v>
       </c>
       <c r="I2" s="2">
-        <v>4.8305930361838938E-2</v>
+        <v>4.6876134153442273E-2</v>
       </c>
       <c r="J2" s="2">
-        <v>6.0563978398811218E-2</v>
+        <v>6.006636732624715E-2</v>
       </c>
       <c r="K2" s="2">
-        <v>5.4000000000000714E-3</v>
+        <v>-9.7000000000000419E-3</v>
       </c>
       <c r="L2" s="2">
-        <v>1.200990175999994E-2</v>
+        <v>1.4365795256000119E-2</v>
       </c>
       <c r="M2" s="2">
-        <v>2.430152000000008E-2</v>
+        <v>1.4365795256000119E-2</v>
       </c>
       <c r="N2" s="2">
-        <v>0.12811202086357379</v>
+        <v>0.1006594426218692</v>
       </c>
       <c r="O2" s="2">
-        <v>4.4101273556386163E-2</v>
+        <v>4.5985483676901362E-2</v>
       </c>
       <c r="P2" s="2">
-        <v>5.5861172034407103E-2</v>
+        <v>5.7058368915306801E-2</v>
       </c>
       <c r="Q2" s="2">
-        <v>4.6042707792446118E-2</v>
+        <v>4.4279449003390647E-2</v>
       </c>
       <c r="R2" s="2">
-        <v>5.4692512195658072E-2</v>
+        <v>5.3996900192045949E-2</v>
       </c>
       <c r="S2" s="2">
         <v>7.110857750516808E-2</v>
@@ -870,7 +870,7 @@
         <v>-3.3133518868777578E-4</v>
       </c>
       <c r="AG2">
-        <v>36562466.039999999</v>
+        <v>36301330.950000003</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
@@ -881,52 +881,52 @@
         <v>27</v>
       </c>
       <c r="C3" s="2">
-        <v>7.5694677419355649E-3</v>
+        <v>1.1945763888889791E-3</v>
       </c>
       <c r="D3" s="2">
-        <v>1.8621651279313811E-2</v>
+        <v>1.9544161845127968E-2</v>
       </c>
       <c r="E3" s="2">
-        <v>1.832769162855663E-2</v>
+        <v>1.9544161845127968E-2</v>
       </c>
       <c r="F3" s="2">
-        <v>8.0680610327928282E-2</v>
+        <v>7.5732318422108147E-2</v>
       </c>
       <c r="G3" s="2">
-        <v>2.7230256420633921E-2</v>
+        <v>3.3042272690110293E-2</v>
       </c>
       <c r="H3" s="2">
-        <v>1.7817799621784539E-2</v>
+        <v>1.7037497289668298E-2</v>
       </c>
       <c r="I3" s="2">
-        <v>1.8794602267146129E-2</v>
+        <v>1.786013745752291E-2</v>
       </c>
       <c r="J3" s="2">
-        <v>4.417193941064701E-2</v>
+        <v>4.4082138868742682E-2</v>
       </c>
       <c r="K3" s="2">
-        <v>7.3000000000000842E-3</v>
+        <v>2.0000000000000022E-3</v>
       </c>
       <c r="L3" s="2">
-        <v>1.970610826000008E-2</v>
+        <v>2.0215197680000019E-2</v>
       </c>
       <c r="M3" s="2">
-        <v>1.8178840000000029E-2</v>
+        <v>2.0215197680000019E-2</v>
       </c>
       <c r="N3" s="2">
-        <v>8.0432383682738307E-2</v>
+        <v>7.6564487321105101E-2</v>
       </c>
       <c r="O3" s="2">
-        <v>2.9775139913844621E-2</v>
+        <v>3.5536843454010203E-2</v>
       </c>
       <c r="P3" s="2">
-        <v>1.8598628207831199E-2</v>
+        <v>1.7954699742264161E-2</v>
       </c>
       <c r="Q3" s="2">
-        <v>1.9438540178987829E-2</v>
+        <v>1.8726063676071329E-2</v>
       </c>
       <c r="R3" s="2">
-        <v>4.1555062232766733E-2</v>
+        <v>4.1503175432556549E-2</v>
       </c>
       <c r="S3" s="2">
         <v>5.1696869975270232E-2</v>
@@ -971,7 +971,7 @@
         <v>1.9121810314036921E-2</v>
       </c>
       <c r="AG3">
-        <v>91652136.950000003</v>
+        <v>92256175.709999993</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
@@ -982,52 +982,52 @@
         <v>29</v>
       </c>
       <c r="C4" s="2">
-        <v>-1.440096652719669E-2</v>
+        <v>-3.7887260504201659E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>1.491630622523221E-2</v>
+        <v>-6.7613746342441994E-3</v>
       </c>
       <c r="E4" s="2">
-        <v>3.2351599341953641E-2</v>
+        <v>-6.7613746342441994E-3</v>
       </c>
       <c r="F4" s="2">
-        <v>0.1784816937470011</v>
+        <v>0.10747436102419949</v>
       </c>
       <c r="G4" s="2">
-        <v>0.1345101867807692</v>
+        <v>0.1184281154008668</v>
       </c>
       <c r="H4" s="2">
-        <v>0.18919176413225</v>
+        <v>0.1924759110367282</v>
       </c>
       <c r="I4" s="2">
-        <v>0.12962592369786541</v>
+        <v>0.12344629350343279</v>
       </c>
       <c r="J4" s="2">
-        <v>9.9983608596376117E-2</v>
+        <v>9.7916033221743914E-2</v>
       </c>
       <c r="K4" s="2">
-        <v>-8.2999999999999741E-3</v>
+        <v>-3.080000000000005E-2</v>
       </c>
       <c r="L4" s="2">
-        <v>7.7621087179999826E-3</v>
+        <v>-5.9036552800006969E-4</v>
       </c>
       <c r="M4" s="2">
-        <v>3.1169659999999991E-2</v>
+        <v>-5.9036552800006969E-4</v>
       </c>
       <c r="N4" s="2">
-        <v>0.23602978614667311</v>
+        <v>0.15733752172095031</v>
       </c>
       <c r="O4" s="2">
-        <v>0.11082720147125411</v>
+        <v>9.8414974336139105E-2</v>
       </c>
       <c r="P4" s="2">
-        <v>0.16652505376055521</v>
+        <v>0.17333381896318539</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.11083044738618431</v>
+        <v>0.1056276388211768</v>
       </c>
       <c r="R4" s="2">
-        <v>6.9222481484886966E-2</v>
+        <v>6.7631197738589943E-2</v>
       </c>
       <c r="S4" s="2">
         <v>0.20300051409891351</v>
@@ -1072,7 +1072,7 @@
         <v>-4.0965727438507897E-2</v>
       </c>
       <c r="AG4">
-        <v>194018918.53999999</v>
+        <v>186211715.16999999</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -1083,52 +1083,52 @@
         <v>31</v>
       </c>
       <c r="C5" s="2">
-        <v>7.918828571428671E-3</v>
+        <v>-9.0119230769231118E-3</v>
       </c>
       <c r="D5" s="2">
-        <v>1.326329810095417E-2</v>
+        <v>2.0449601669698451E-2</v>
       </c>
       <c r="E5" s="2">
-        <v>2.9729444210970572E-2</v>
+        <v>2.0449601669698451E-2</v>
       </c>
       <c r="F5" s="2">
-        <v>0.18330786302476729</v>
+        <v>0.13595271102089471</v>
       </c>
       <c r="G5" s="2">
-        <v>8.3112735414645256E-2</v>
+        <v>8.2214642489835565E-2</v>
       </c>
       <c r="H5" s="2">
-        <v>0.1064525704765933</v>
+        <v>0.1139290118596934</v>
       </c>
       <c r="I5" s="2">
-        <v>6.7864542774802139E-2</v>
+        <v>6.5610391484684616E-2</v>
       </c>
       <c r="J5" s="2">
-        <v>7.785440782670916E-2</v>
+        <v>7.7280936573876025E-2</v>
       </c>
       <c r="K5" s="2">
-        <v>2.0000000000000022E-3</v>
+        <v>-1.019999999999999E-2</v>
       </c>
       <c r="L5" s="2">
-        <v>4.729768640000076E-3</v>
+        <v>1.726833572000008E-2</v>
       </c>
       <c r="M5" s="2">
-        <v>2.7751400000000089E-2</v>
+        <v>1.726833572000008E-2</v>
       </c>
       <c r="N5" s="2">
-        <v>0.16749776863039581</v>
+        <v>0.12542782566260799</v>
       </c>
       <c r="O5" s="2">
-        <v>6.0813720199518473E-2</v>
+        <v>5.778076241459229E-2</v>
       </c>
       <c r="P5" s="2">
-        <v>9.6550005519527415E-2</v>
+        <v>0.1035994179696009</v>
       </c>
       <c r="Q5" s="2">
-        <v>6.2541536792744656E-2</v>
+        <v>6.0336104317869843E-2</v>
       </c>
       <c r="R5" s="2">
-        <v>7.471156024925496E-2</v>
+        <v>7.4104034579170364E-2</v>
       </c>
       <c r="S5" s="2">
         <v>0.16909176936559361</v>
@@ -1173,7 +1173,7 @@
         <v>-4.6556803672422993E-2</v>
       </c>
       <c r="AG5">
-        <v>18275998.289999999</v>
+        <v>18333995.43</v>
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
@@ -1184,52 +1184,52 @@
         <v>33</v>
       </c>
       <c r="C6" s="2">
-        <v>5.9103846153845119E-3</v>
+        <v>-1.210428571428568E-2</v>
       </c>
       <c r="D6" s="2">
-        <v>8.8847202734911868E-3</v>
+        <v>1.864060358322717E-2</v>
       </c>
       <c r="E6" s="2">
-        <v>3.1121593962721631E-2</v>
+        <v>1.864060358322717E-2</v>
       </c>
       <c r="F6" s="2">
-        <v>0.24024368450940181</v>
+        <v>0.16844499389353601</v>
       </c>
       <c r="G6" s="2">
-        <v>0.11819146980306169</v>
+        <v>0.1121131986151627</v>
       </c>
       <c r="H6" s="2">
-        <v>0.1586984910917506</v>
+        <v>0.17394038629166131</v>
       </c>
       <c r="I6" s="2">
-        <v>9.1123660866985423E-2</v>
+        <v>8.8567757119815571E-2</v>
       </c>
       <c r="J6" s="2">
-        <v>8.5615166196782777E-2</v>
+        <v>8.4884353051230654E-2</v>
       </c>
       <c r="K6" s="2">
-        <v>-4.0000000000000044E-3</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L6" s="2">
-        <v>-3.041808160000103E-3</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M6" s="2">
-        <v>3.0660799999999929E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N6" s="2">
-        <v>0.22454925336440401</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O6" s="2">
-        <v>8.844086955805297E-2</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P6" s="2">
-        <v>0.1534472761844223</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q6" s="2">
-        <v>8.8153012204149617E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R6" s="2">
-        <v>7.5294552309795204E-2</v>
+        <v>7.448544676534663E-2</v>
       </c>
       <c r="S6" s="2">
         <v>0.2464799745561268</v>
@@ -1274,7 +1274,7 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG6">
-        <v>21148869.02</v>
+        <v>22622943.23</v>
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
@@ -1285,52 +1285,52 @@
         <v>35</v>
       </c>
       <c r="C7" s="2">
-        <v>1.2121467391304369E-2</v>
+        <v>-3.418017543859619E-3</v>
       </c>
       <c r="D7" s="2">
-        <v>1.8894675461928578E-2</v>
+        <v>2.198868032147927E-2</v>
       </c>
       <c r="E7" s="2">
-        <v>2.5493836244884219E-2</v>
+        <v>2.198868032147927E-2</v>
       </c>
       <c r="F7" s="2">
-        <v>9.3862884628607812E-2</v>
+        <v>8.3191615757522097E-2</v>
       </c>
       <c r="G7" s="2">
-        <v>2.0995220498161379E-2</v>
+        <v>2.8382404312901951E-2</v>
       </c>
       <c r="H7" s="2">
-        <v>1.4327082069022451E-2</v>
+        <v>1.226898501527063E-2</v>
       </c>
       <c r="I7" s="2">
-        <v>2.09171157542416E-2</v>
+        <v>1.9178763704715381E-2</v>
       </c>
       <c r="J7" s="2">
-        <v>5.2740659169707722E-2</v>
+        <v>5.2481061802177598E-2</v>
       </c>
       <c r="K7" s="2">
-        <v>1.09999999999999E-2</v>
+        <v>-2.8000000000000251E-3</v>
       </c>
       <c r="L7" s="2">
-        <v>1.607238919999987E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="M7" s="2">
-        <v>2.313199999999993E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="N7" s="2">
-        <v>8.4867214211104436E-2</v>
+        <v>7.6447349264987974E-2</v>
       </c>
       <c r="O7" s="2">
-        <v>1.6559852705851918E-2</v>
+        <v>2.379636305646082E-2</v>
       </c>
       <c r="P7" s="2">
-        <v>9.6988969437727945E-3</v>
+        <v>8.0919721626715457E-3</v>
       </c>
       <c r="Q7" s="2">
-        <v>1.8966073465605641E-2</v>
+        <v>1.7300619327857539E-2</v>
       </c>
       <c r="R7" s="2">
-        <v>5.1124428236377861E-2</v>
+        <v>5.0890382612324807E-2</v>
       </c>
       <c r="S7" s="2">
         <v>4.9758392035209147E-2</v>
@@ -1375,7 +1375,7 @@
         <v>1.4079379818825901E-2</v>
       </c>
       <c r="AG7">
-        <v>91233383.430000007</v>
+        <v>90357940.280000001</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
@@ -1386,52 +1386,52 @@
         <v>37</v>
       </c>
       <c r="C8" s="2">
-        <v>-5.3746141732283759E-3</v>
+        <v>-3.1215904411764691E-2</v>
       </c>
       <c r="D8" s="2">
-        <v>4.5854165693122402E-2</v>
+        <v>5.7615191611672936E-3</v>
       </c>
       <c r="E8" s="2">
-        <v>3.8168900316720933E-2</v>
+        <v>5.7615191611672936E-3</v>
       </c>
       <c r="F8" s="2">
-        <v>0.21379324138002501</v>
+        <v>0.15602004284453441</v>
       </c>
       <c r="G8" s="2">
-        <v>0.13632166281808281</v>
+        <v>0.13273323400015791</v>
       </c>
       <c r="H8" s="2">
-        <v>0.15509314804414381</v>
+        <v>0.1551478095151588</v>
       </c>
       <c r="I8" s="2">
-        <v>0.11435879204735989</v>
+        <v>0.10734378244820771</v>
       </c>
       <c r="J8" s="2">
-        <v>0.1062437853248233</v>
+        <v>0.10425048159546151</v>
       </c>
       <c r="K8" s="2">
-        <v>-1.2499999999999961E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L8" s="2">
-        <v>2.9880537499999971E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M8" s="2">
-        <v>2.9468749999999929E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N8" s="2">
-        <v>0.2279335112320855</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O8" s="2">
-        <v>0.1406458000440951</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P8" s="2">
-        <v>0.1663213492098834</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.12248757151155699</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R8" s="2">
-        <v>9.4006958248271877E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="S8" s="2">
         <v>0.25956354944849203</v>
@@ -1476,7 +1476,7 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG8">
-        <v>122618881.38</v>
+        <v>122930009.13</v>
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
@@ -1487,52 +1487,52 @@
         <v>37</v>
       </c>
       <c r="C9" s="2">
-        <v>-7.6082558139535239E-3</v>
+        <v>-3.5942372093023311E-2</v>
       </c>
       <c r="D9" s="2">
-        <v>4.13274011843483E-2</v>
+        <v>-6.235734338472243E-4</v>
       </c>
       <c r="E9" s="2">
-        <v>3.6635567871450947E-2</v>
+        <v>-6.235734338472243E-4</v>
       </c>
       <c r="F9" s="2">
-        <v>0.21448341747325911</v>
+        <v>0.1517135575266855</v>
       </c>
       <c r="G9" s="2">
-        <v>0.13775310599180979</v>
+        <v>0.13471849448114859</v>
       </c>
       <c r="H9" s="2">
-        <v>0.16183008748527139</v>
+        <v>0.16098799855349261</v>
       </c>
       <c r="I9" s="2">
-        <v>0.1175711466571818</v>
+        <v>0.1097896375134306</v>
       </c>
       <c r="J9" s="2">
-        <v>9.0977203684160513E-2</v>
+        <v>8.820677654857545E-2</v>
       </c>
       <c r="K9" s="2">
-        <v>-1.2499999999999961E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L9" s="2">
-        <v>2.9880537499999971E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M9" s="2">
-        <v>2.9468749999999929E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N9" s="2">
-        <v>0.2279335112320855</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O9" s="2">
-        <v>0.1406458000440951</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P9" s="2">
-        <v>0.1663213492098834</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q9" s="2">
-        <v>0.12248757151155699</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R9" s="2">
-        <v>0.1011815742271851</v>
+        <v>9.7708296429523944E-2</v>
       </c>
       <c r="S9" s="2">
         <v>0.26275886187340619</v>
@@ -1577,7 +1577,7 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG9">
-        <v>39805919.340000004</v>
+        <v>39123712.670000002</v>
       </c>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.25">
@@ -1588,52 +1588,52 @@
         <v>40</v>
       </c>
       <c r="C10" s="2">
-        <v>1.8945222222222169E-2</v>
+        <v>6.3950454545453894E-3</v>
       </c>
       <c r="D10" s="2">
-        <v>7.2532924185209069E-3</v>
+        <v>5.1071890506063873E-2</v>
       </c>
       <c r="E10" s="2">
-        <v>4.4392950117654761E-2</v>
+        <v>5.1071890506063873E-2</v>
       </c>
       <c r="F10" s="2">
-        <v>0.18009142345083079</v>
+        <v>0.13703988678249709</v>
       </c>
       <c r="G10" s="2">
-        <v>8.679407272750117E-2</v>
+        <v>7.7785554375998434E-2</v>
       </c>
       <c r="H10" s="2">
-        <v>0.14945988183847941</v>
+        <v>0.1716444837461153</v>
       </c>
       <c r="I10" s="2">
-        <v>7.8806861055847222E-2</v>
+        <v>7.875779031571617E-2</v>
       </c>
       <c r="J10" s="2">
-        <v>0.11308402972963801</v>
+        <v>0.1129563102030335</v>
       </c>
       <c r="K10" s="2">
-        <v>7.3000000000000842E-3</v>
+        <v>4.8999999999999044E-3</v>
       </c>
       <c r="L10" s="2">
-        <v>-9.5969337039998326E-3</v>
+        <v>2.9646225244000179E-2</v>
       </c>
       <c r="M10" s="2">
-        <v>2.4625560000000268E-2</v>
+        <v>2.9646225244000179E-2</v>
       </c>
       <c r="N10" s="2">
-        <v>0.17748268133895739</v>
+        <v>0.1415845117969303</v>
       </c>
       <c r="O10" s="2">
-        <v>6.2201389485577741E-2</v>
+        <v>5.1073641533631919E-2</v>
       </c>
       <c r="P10" s="2">
-        <v>0.15014573708926321</v>
+        <v>0.1761650828228889</v>
       </c>
       <c r="Q10" s="2">
-        <v>7.9416698848171485E-2</v>
+        <v>7.97362843438989E-2</v>
       </c>
       <c r="R10" s="2">
-        <v>0.1064120381222424</v>
+        <v>0.106236078843726</v>
       </c>
       <c r="S10" s="2">
         <v>0.13308185228320671</v>
@@ -1678,7 +1678,7 @@
         <v>-0.107731401591228</v>
       </c>
       <c r="AG10">
-        <v>12875041.279999999</v>
+        <v>12959685.77</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.25">
@@ -1689,52 +1689,52 @@
         <v>42</v>
       </c>
       <c r="C11" s="2">
-        <v>-1.3420137254901991E-2</v>
+        <v>-2.793517094017095E-2</v>
       </c>
       <c r="D11" s="2">
-        <v>8.140361089503223E-3</v>
+        <v>-6.9974686044145251E-3</v>
       </c>
       <c r="E11" s="2">
-        <v>2.153940941985022E-2</v>
+        <v>-6.9974686044145251E-3</v>
       </c>
       <c r="F11" s="2">
-        <v>0.1600602187976301</v>
+        <v>0.11055124904926709</v>
       </c>
       <c r="G11" s="2">
-        <v>9.0287993205319772E-2</v>
+        <v>8.8926692211731106E-2</v>
       </c>
       <c r="H11" s="2">
-        <v>0.10381088748291489</v>
+        <v>0.1042701786341529</v>
       </c>
       <c r="I11" s="2">
-        <v>7.7911945543049477E-2</v>
+        <v>7.2921934057077031E-2</v>
       </c>
       <c r="J11" s="2">
-        <v>7.8496357094812064E-2</v>
+        <v>7.7175098624535421E-2</v>
       </c>
       <c r="K11" s="2">
-        <v>-9.9999999999988987E-5</v>
+        <v>-1.9499999999999958E-2</v>
       </c>
       <c r="L11" s="2">
-        <v>1.204138573999991E-2</v>
+        <v>3.343355630000211E-3</v>
       </c>
       <c r="M11" s="2">
-        <v>2.3297660000000109E-2</v>
+        <v>3.343355630000211E-3</v>
       </c>
       <c r="N11" s="2">
-        <v>0.16155697124099541</v>
+        <v>0.1162468002565875</v>
       </c>
       <c r="O11" s="2">
-        <v>7.0034058988779124E-2</v>
+        <v>6.7799862845294712E-2</v>
       </c>
       <c r="P11" s="2">
-        <v>9.0777320025655195E-2</v>
+        <v>9.2129731790285385E-2</v>
       </c>
       <c r="Q11" s="2">
-        <v>6.9785817526893723E-2</v>
+        <v>6.5838927258658142E-2</v>
       </c>
       <c r="R11" s="2">
-        <v>7.1317974567514097E-2</v>
+        <v>7.0353902482109154E-2</v>
       </c>
       <c r="S11" s="2">
         <v>0.18322548414762951</v>
@@ -1779,7 +1779,7 @@
         <v>-6.1622847520066406E-3</v>
       </c>
       <c r="AG11">
-        <v>106782884.31999999</v>
+        <v>103905181.66</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.25">
@@ -1790,52 +1790,52 @@
         <v>44</v>
       </c>
       <c r="C12" s="2">
-        <v>-2.7202454545454561E-2</v>
+        <v>-4.4305312500000027E-2</v>
       </c>
       <c r="D12" s="2">
-        <v>4.139584885668901E-3</v>
+        <v>-2.277153520861519E-2</v>
       </c>
       <c r="E12" s="2">
-        <v>2.2532067587102581E-2</v>
+        <v>-2.277153520861519E-2</v>
       </c>
       <c r="F12" s="2">
-        <v>0.21482190052553299</v>
+        <v>0.1417040383429102</v>
       </c>
       <c r="G12" s="2">
-        <v>0.14321177678706659</v>
+        <v>0.13551532035802749</v>
       </c>
       <c r="H12" s="2">
-        <v>0.16398219118923299</v>
+        <v>0.1655807769124944</v>
       </c>
       <c r="I12" s="2">
-        <v>0.11228653030534549</v>
+        <v>0.1049735988515956</v>
       </c>
       <c r="J12" s="2">
-        <v>0.1027610864985045</v>
+        <v>0.10067588666941329</v>
       </c>
       <c r="K12" s="2">
-        <v>-1.1199999999999989E-2</v>
+        <v>-3.6100000000000021E-2</v>
       </c>
       <c r="L12" s="2">
-        <v>7.9594831999998394E-3</v>
+        <v>-1.363233923200002E-2</v>
       </c>
       <c r="M12" s="2">
-        <v>2.3309119999999961E-2</v>
+        <v>-1.363233923200002E-2</v>
       </c>
       <c r="N12" s="2">
-        <v>0.242032551733292</v>
+        <v>0.15604014736937091</v>
       </c>
       <c r="O12" s="2">
-        <v>0.1252717903859055</v>
+        <v>0.1127104918208743</v>
       </c>
       <c r="P12" s="2">
-        <v>0.17458595810543279</v>
+        <v>0.1800864836126552</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.1200798665158682</v>
+        <v>0.1136342374131081</v>
       </c>
       <c r="R12" s="2">
-        <v>9.0552237365185695E-2</v>
+        <v>8.8855331373153934E-2</v>
       </c>
       <c r="S12" s="2">
         <v>0.28821327176199668</v>
@@ -1880,7 +1880,7 @@
         <v>-2.4421037083545372E-2</v>
       </c>
       <c r="AG12">
-        <v>37499681.399999999</v>
+        <v>36094359.75</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
@@ -1891,52 +1891,52 @@
         <v>46</v>
       </c>
       <c r="C13" s="2">
-        <v>-4.4192049180327819E-2</v>
+        <v>-6.7599536231884083E-2</v>
       </c>
       <c r="D13" s="2">
-        <v>-2.6737882786119771E-3</v>
+        <v>-6.031086254876461E-2</v>
       </c>
       <c r="E13" s="2">
-        <v>7.8171064540912827E-3</v>
+        <v>-6.031086254876461E-2</v>
       </c>
       <c r="F13" s="2">
-        <v>0.18381795671660581</v>
+        <v>8.5448334998118547E-2</v>
       </c>
       <c r="G13" s="2">
-        <v>0.1265569932867503</v>
+        <v>0.1101392932249632</v>
       </c>
       <c r="H13" s="2">
-        <v>0.18147028888424499</v>
+        <v>0.1717278808634366</v>
       </c>
       <c r="I13" s="2">
-        <v>0.14516575586870251</v>
+        <v>0.13358848677320401</v>
       </c>
       <c r="J13" s="2">
-        <v>0.1000872749936903</v>
+        <v>9.662836043779599E-2</v>
       </c>
       <c r="K13" s="2">
-        <v>-1.8299999999999979E-2</v>
+        <v>-5.7200000000000029E-2</v>
       </c>
       <c r="L13" s="2">
-        <v>1.8802860649999701E-2</v>
+        <v>-4.2059103400000082E-2</v>
       </c>
       <c r="M13" s="2">
-        <v>1.605949999999989E-2</v>
+        <v>-4.2059103400000082E-2</v>
       </c>
       <c r="N13" s="2">
-        <v>0.25764938941815968</v>
+        <v>0.1514001207452329</v>
       </c>
       <c r="O13" s="2">
-        <v>0.1583162539418059</v>
+        <v>0.1431775036972347</v>
       </c>
       <c r="P13" s="2">
-        <v>0.19217134054854479</v>
+        <v>0.18839266096490029</v>
       </c>
       <c r="Q13" s="2">
-        <v>0.14946663466863039</v>
+        <v>0.13895702040647101</v>
       </c>
       <c r="R13" s="2">
-        <v>7.5641001525709406E-2</v>
+        <v>7.2820767080817639E-2</v>
       </c>
       <c r="S13" s="2">
         <v>0.27366522335215349</v>
@@ -1981,7 +1981,7 @@
         <v>4.2275010225730332E-2</v>
       </c>
       <c r="AG13">
-        <v>63175036.729999997</v>
+        <v>58597796.509999998</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
@@ -1992,52 +1992,52 @@
         <v>33</v>
       </c>
       <c r="C14" s="2">
-        <v>-4.7083781512604617E-3</v>
+        <v>-2.2661366906474578E-3</v>
       </c>
       <c r="D14" s="2">
-        <v>-8.3803026289983595E-3</v>
+        <v>1.116373208500754E-2</v>
       </c>
       <c r="E14" s="2">
-        <v>1.346037181810167E-2</v>
+        <v>1.116373208500754E-2</v>
       </c>
       <c r="F14" s="2">
-        <v>0.15895056324829479</v>
+        <v>0.13099004582773069</v>
       </c>
       <c r="G14" s="2">
-        <v>8.9560796014035438E-2</v>
+        <v>8.2063146975251744E-2</v>
       </c>
       <c r="H14" s="2">
-        <v>0.15131163075430359</v>
+        <v>0.17067287764213049</v>
       </c>
       <c r="I14" s="2">
-        <v>7.9066382825266457E-2</v>
+        <v>7.8035810823603002E-2</v>
       </c>
       <c r="J14" s="2">
-        <v>0.117651463165463</v>
+        <v>0.1171603222233009</v>
       </c>
       <c r="K14" s="2">
-        <v>-4.0000000000000044E-3</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L14" s="2">
-        <v>-3.041808160000103E-3</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M14" s="2">
-        <v>3.0660799999999929E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N14" s="2">
-        <v>0.22454925336440401</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O14" s="2">
-        <v>8.844086955805297E-2</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P14" s="2">
-        <v>0.1534472761844223</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q14" s="2">
-        <v>8.8153012204149617E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R14" s="2">
-        <v>8.1277551446557572E-2</v>
+        <v>8.0382949158205319E-2</v>
       </c>
       <c r="S14" s="2">
         <v>0.19391940521041101</v>
@@ -2082,7 +2082,7 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG14">
-        <v>100366932.59</v>
+        <v>101817758.04000001</v>
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.25">
@@ -2093,52 +2093,52 @@
         <v>49</v>
       </c>
       <c r="C15" s="2">
-        <v>-2.7122199999999989E-2</v>
+        <v>-9.1109999999999802E-3</v>
       </c>
       <c r="D15" s="2">
-        <v>1.3133811032997929E-2</v>
+        <v>1.9400413770960471E-2</v>
       </c>
       <c r="E15" s="2">
-        <v>2.877356976509016E-2</v>
+        <v>1.9400413770960471E-2</v>
       </c>
       <c r="F15" s="2">
-        <v>0.14963819388483299</v>
+        <v>0.1241008883958441</v>
       </c>
       <c r="G15" s="2">
-        <v>9.5605664391316791E-2</v>
+        <v>8.8651462309059736E-2</v>
       </c>
       <c r="H15" s="2">
-        <v>0.17091819024024679</v>
+        <v>0.19512163393811791</v>
       </c>
       <c r="I15" s="2">
-        <v>8.983680290657281E-2</v>
+        <v>8.881798785427919E-2</v>
       </c>
       <c r="J15" s="2">
-        <v>0.1127018313800365</v>
+        <v>0.1119716522842138</v>
       </c>
       <c r="K15" s="2">
-        <v>-2.270000000000005E-2</v>
+        <v>2.5600000000000071E-2</v>
       </c>
       <c r="L15" s="2">
-        <v>-4.8808080850000102E-2</v>
+        <v>8.8339527199998713E-3</v>
       </c>
       <c r="M15" s="2">
-        <v>-1.63475500000001E-2</v>
+        <v>8.8339527199998713E-3</v>
       </c>
       <c r="N15" s="2">
-        <v>0.16415145540221809</v>
+        <v>0.1107579613550238</v>
       </c>
       <c r="O15" s="2">
-        <v>1.7771351911434641E-2</v>
+        <v>1.877174809602411E-2</v>
       </c>
       <c r="P15" s="2">
-        <v>0.16268018594929259</v>
+        <v>0.2041523735077295</v>
       </c>
       <c r="Q15" s="2">
-        <v>6.6691636391552844E-2</v>
+        <v>6.9387845268587434E-2</v>
       </c>
       <c r="R15" s="2">
-        <v>6.1561346956535479E-2</v>
+        <v>6.2345238662887333E-2</v>
       </c>
       <c r="S15" s="2">
         <v>0.1454564677544905</v>
@@ -2183,7 +2183,7 @@
         <v>-0.18167452986828991</v>
       </c>
       <c r="AG15">
-        <v>15122269.26</v>
+        <v>15321258.43</v>
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.25">
@@ -2194,52 +2194,52 @@
         <v>33</v>
       </c>
       <c r="C16" s="2">
-        <v>-1.0710000000000001E-2</v>
+        <v>-2.0684363636363608E-2</v>
       </c>
       <c r="D16" s="2">
-        <v>-2.350010568781935E-2</v>
+        <v>-1.219021590950875E-2</v>
       </c>
       <c r="E16" s="2">
-        <v>8.6735546859999513E-3</v>
+        <v>-1.219021590950875E-2</v>
       </c>
       <c r="F16" s="2">
-        <v>0.16476171868558559</v>
+        <v>0.10316186048992</v>
       </c>
       <c r="G16" s="2">
-        <v>8.1191072392124308E-2</v>
+        <v>6.4476624925824622E-2</v>
       </c>
       <c r="H16" s="2">
-        <v>0.16115318539571</v>
+        <v>0.17601504224335079</v>
       </c>
       <c r="I16" s="2">
-        <v>9.5629547620493138E-2</v>
+        <v>9.302266890190003E-2</v>
       </c>
       <c r="J16" s="2">
-        <v>9.6931216298767886E-2</v>
+        <v>9.5820830509585564E-2</v>
       </c>
       <c r="K16" s="2">
-        <v>-4.0000000000000044E-3</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L16" s="2">
-        <v>-3.041808160000103E-3</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M16" s="2">
-        <v>3.0660799999999929E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N16" s="2">
-        <v>0.22454925336440401</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O16" s="2">
-        <v>8.844086955805297E-2</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P16" s="2">
-        <v>0.1534472761844223</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q16" s="2">
-        <v>8.8153012204149617E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R16" s="2">
-        <v>7.5294552309795204E-2</v>
+        <v>7.448544676534663E-2</v>
       </c>
       <c r="S16" s="2">
         <v>0.1789907355690501</v>
@@ -2284,7 +2284,7 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG16">
-        <v>5253093.3</v>
+        <v>5275300.41</v>
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.25">
@@ -2295,52 +2295,52 @@
         <v>52</v>
       </c>
       <c r="C17" s="2">
-        <v>-2.3705708333333301E-2</v>
+        <v>-5.0939892857142843E-2</v>
       </c>
       <c r="D17" s="2">
-        <v>2.4300625670954371E-2</v>
+        <v>-2.8692617988143269E-2</v>
       </c>
       <c r="E17" s="2">
-        <v>2.344137605359364E-2</v>
+        <v>-2.8692617988143269E-2</v>
       </c>
       <c r="F17" s="2">
-        <v>0.14150176970463829</v>
+        <v>6.7028259489456454E-2</v>
       </c>
       <c r="G17" s="2">
-        <v>9.6726345575876893E-2</v>
+        <v>9.088803846271909E-2</v>
       </c>
       <c r="H17" s="2">
-        <v>0.12530952665806391</v>
+        <v>0.1224068762633332</v>
       </c>
       <c r="I17" s="2">
-        <v>0.10596760780018059</v>
+        <v>9.5909508957356282E-2</v>
       </c>
       <c r="J17" s="2">
-        <v>8.2773748212795484E-2</v>
+        <v>7.9910729147968595E-2</v>
       </c>
       <c r="K17" s="2">
-        <v>-1.129999999999998E-2</v>
+        <v>-4.0399999999999991E-2</v>
       </c>
       <c r="L17" s="2">
-        <v>3.2023172983999697E-2</v>
+        <v>-1.25342139839999E-2</v>
       </c>
       <c r="M17" s="2">
-        <v>2.9038960000000062E-2</v>
+        <v>-1.25342139839999E-2</v>
       </c>
       <c r="N17" s="2">
-        <v>0.22217808931760799</v>
+        <v>0.1397493629826794</v>
       </c>
       <c r="O17" s="2">
-        <v>0.1285784993239765</v>
+        <v>0.12140449706502079</v>
       </c>
       <c r="P17" s="2">
-        <v>0.1515182028381199</v>
+        <v>0.15465495678796759</v>
       </c>
       <c r="Q17" s="2">
-        <v>0.10932933684393251</v>
+        <v>0.1006417652541247</v>
       </c>
       <c r="R17" s="2">
-        <v>8.2549190928752791E-2</v>
+        <v>8.0223669909337936E-2</v>
       </c>
       <c r="S17" s="2">
         <v>0.19251440061512121</v>
@@ -2385,7 +2385,7 @@
         <v>-1.2569244036318761E-2</v>
       </c>
       <c r="AG17">
-        <v>28973759.07</v>
+        <v>27474507.350000001</v>
       </c>
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.25">
@@ -2396,52 +2396,52 @@
         <v>54</v>
       </c>
       <c r="C18" s="2">
-        <v>8.2566551724136961E-3</v>
+        <v>-2.9110799999999989E-2</v>
       </c>
       <c r="D18" s="2">
-        <v>6.9968365460913562E-2</v>
+        <v>4.6301933509756532E-2</v>
       </c>
       <c r="E18" s="2">
-        <v>7.7673882364492908E-2</v>
+        <v>4.6301933509756532E-2</v>
       </c>
       <c r="F18" s="2">
-        <v>0.1408914004992097</v>
+        <v>7.6880360798713854E-2</v>
       </c>
       <c r="G18" s="2">
-        <v>9.6323739561103183E-2</v>
+        <v>9.8296011522881477E-2</v>
       </c>
       <c r="H18" s="2">
-        <v>9.6970367994610562E-2</v>
+        <v>0.10389964249085031</v>
       </c>
       <c r="I18" s="2">
-        <v>6.3852103991039577E-2</v>
+        <v>5.8994578820060761E-2</v>
       </c>
       <c r="J18" s="2">
-        <v>6.7415623409172509E-2</v>
+        <v>6.4242663443119241E-2</v>
       </c>
       <c r="K18" s="2">
-        <v>1.3700000000000051E-2</v>
+        <v>-3.800000000000026E-3</v>
       </c>
       <c r="L18" s="2">
-        <v>7.913111143400009E-2</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="M18" s="2">
-        <v>7.4724740000000178E-2</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="N18" s="2">
-        <v>0.16088398918518679</v>
+        <v>0.1209388679134276</v>
       </c>
       <c r="O18" s="2">
-        <v>0.1100918047856789</v>
+        <v>0.1174481059475172</v>
       </c>
       <c r="P18" s="2">
-        <v>0.1128371284909728</v>
+        <v>0.12467008367003379</v>
       </c>
       <c r="Q18" s="2">
-        <v>7.3560596447728166E-2</v>
+        <v>7.144945945259229E-2</v>
       </c>
       <c r="R18" s="2">
-        <v>7.6153486414625826E-2</v>
+        <v>7.524501681840956E-2</v>
       </c>
       <c r="S18" s="2">
         <v>0.1238325144064758</v>
@@ -2486,7 +2486,7 @@
         <v>-5.5537819245731417E-2</v>
       </c>
       <c r="AG18">
-        <v>20320475.079999998</v>
+        <v>18788911.550000001</v>
       </c>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.25">
@@ -2497,52 +2497,52 @@
         <v>33</v>
       </c>
       <c r="C19" s="2">
-        <v>-3.1554166666666328E-3</v>
+        <v>3.9472499999999577E-3</v>
       </c>
       <c r="D19" s="2">
-        <v>4.8339672149866342E-3</v>
+        <v>3.2863056265764801E-2</v>
       </c>
       <c r="E19" s="2">
-        <v>2.8802117109006261E-2</v>
+        <v>3.2863056265764801E-2</v>
       </c>
       <c r="F19" s="2">
-        <v>0.17157620436662491</v>
+        <v>0.15054358655904451</v>
       </c>
       <c r="G19" s="2">
-        <v>0.1022847200262036</v>
+        <v>9.1249189552183418E-2</v>
       </c>
       <c r="H19" s="2">
-        <v>0.15971397231577281</v>
+        <v>0.1819130928844486</v>
       </c>
       <c r="I19" s="2">
-        <v>8.9002833803629278E-2</v>
+        <v>8.8295704973029299E-2</v>
       </c>
       <c r="J19" s="2">
-        <v>8.6420627476248457E-2</v>
+        <v>8.6261410546911721E-2</v>
       </c>
       <c r="K19" s="2">
-        <v>-4.0000000000000044E-3</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L19" s="2">
-        <v>-3.041808160000103E-3</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M19" s="2">
-        <v>3.0660799999999929E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N19" s="2">
-        <v>0.22454925336440401</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O19" s="2">
-        <v>8.844086955805297E-2</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P19" s="2">
-        <v>0.1534472761844223</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q19" s="2">
-        <v>8.8153012204149617E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R19" s="2">
-        <v>8.2190923454147802E-2</v>
+        <v>8.1026660239410964E-2</v>
       </c>
       <c r="S19" s="2">
         <v>0.17063771874488459</v>
@@ -2587,7 +2587,7 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG19">
-        <v>6349880.5800000001</v>
+        <v>4214482.78</v>
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
@@ -2598,52 +2598,52 @@
         <v>33</v>
       </c>
       <c r="C20" s="2">
-        <v>4.8459999999999059E-3</v>
+        <v>-2.1749600000000039E-2</v>
       </c>
       <c r="D20" s="2">
-        <v>-7.8954830360582484E-3</v>
+        <v>9.9861952172015656E-3</v>
       </c>
       <c r="E20" s="2">
-        <v>3.2441382305799848E-2</v>
+        <v>9.9861952172015656E-3</v>
       </c>
       <c r="F20" s="2">
-        <v>0.21393152861939951</v>
+        <v>0.1318423593638387</v>
       </c>
       <c r="G20" s="2">
-        <v>0.11153940092618921</v>
+        <v>9.8240397167722815E-2</v>
       </c>
       <c r="H20" s="2">
-        <v>0.13183699266832849</v>
+        <v>0.16899659813090301</v>
       </c>
       <c r="I20" s="2">
-        <v>8.8114418446086917E-2</v>
+        <v>8.7613179492281423E-2</v>
       </c>
       <c r="J20" s="2">
-        <v>8.5032396039284919E-2</v>
+        <v>8.2816539945535839E-2</v>
       </c>
       <c r="K20" s="2">
-        <v>-4.0000000000000044E-3</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L20" s="2">
-        <v>-3.041808160000103E-3</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M20" s="2">
-        <v>3.0660799999999929E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N20" s="2">
-        <v>0.22454925336440401</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O20" s="2">
-        <v>8.844086955805297E-2</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1534472761844223</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q20" s="2">
-        <v>8.8153012204149617E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R20" s="2">
-        <v>7.6009339007235388E-2</v>
+        <v>7.4381651558945938E-2</v>
       </c>
       <c r="S20" s="2">
         <v>0.21693517822200331</v>
@@ -2688,7 +2688,7 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG20">
-        <v>11712856.67</v>
+        <v>11633336.32</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
@@ -2699,52 +2699,52 @@
         <v>35</v>
       </c>
       <c r="C21" s="2">
-        <v>1.324039999999993E-2</v>
+        <v>-2.1986999999999979E-3</v>
       </c>
       <c r="D21" s="2">
-        <v>1.897525914572951E-2</v>
+        <v>2.366803950823115E-2</v>
       </c>
       <c r="E21" s="2">
-        <v>2.5923738031039981E-2</v>
+        <v>2.366803950823115E-2</v>
       </c>
       <c r="F21" s="2">
-        <v>9.3551183475714561E-2</v>
+        <v>8.4854635602114037E-2</v>
       </c>
       <c r="G21" s="2">
-        <v>2.010687257659249E-2</v>
+        <v>3.029970404733762E-2</v>
       </c>
       <c r="H21" s="2">
-        <v>1.0488623387680199E-2</v>
+        <v>1.0661860433113681E-2</v>
       </c>
       <c r="I21" s="2">
-        <v>2.2752768678667271E-2</v>
+        <v>2.2844225768598129E-2</v>
       </c>
       <c r="J21" s="2">
-        <v>2.8516004411741399E-2</v>
+        <v>2.8184191500508989E-2</v>
       </c>
       <c r="K21" s="2">
-        <v>1.09999999999999E-2</v>
+        <v>-2.8000000000000251E-3</v>
       </c>
       <c r="L21" s="2">
-        <v>1.607238919999987E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="M21" s="2">
-        <v>2.313199999999993E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="N21" s="2">
-        <v>8.4867214211104436E-2</v>
+        <v>7.6447349264987974E-2</v>
       </c>
       <c r="O21" s="2">
-        <v>1.6559852705851918E-2</v>
+        <v>2.379636305646082E-2</v>
       </c>
       <c r="P21" s="2">
-        <v>9.6988969437727945E-3</v>
+        <v>8.0919721626715457E-3</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.8966073465605641E-2</v>
+        <v>1.7300619327857539E-2</v>
       </c>
       <c r="R21" s="2">
-        <v>3.02405208241141E-2</v>
+        <v>2.985386050536731E-2</v>
       </c>
       <c r="S21" s="2">
         <v>4.7779083879743611E-2</v>
@@ -2789,7 +2789,7 @@
         <v>1.4079379818825901E-2</v>
       </c>
       <c r="AG21">
-        <v>14267134.48</v>
+        <v>14289819.52</v>
       </c>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
@@ -2800,52 +2800,52 @@
         <v>59</v>
       </c>
       <c r="C22" s="2">
-        <v>-2.6336000000000141E-3</v>
+        <v>-1.805699999999999E-2</v>
       </c>
       <c r="D22" s="2">
-        <v>1.397849875872903E-2</v>
+        <v>3.0886347110097301E-3</v>
       </c>
       <c r="E22" s="2">
-        <v>2.1534482868160069E-2</v>
+        <v>3.0886347110097301E-3</v>
       </c>
       <c r="F22" s="2">
-        <v>0.1692093334857572</v>
+        <v>0.1247030961510633</v>
       </c>
       <c r="G22" s="2">
-        <v>9.3698566827340679E-2</v>
+        <v>8.6284729443472763E-2</v>
       </c>
       <c r="H22" s="2">
-        <v>0.12639633226276409</v>
+        <v>0.1396859127128007</v>
       </c>
       <c r="I22" s="2">
-        <v>8.5653959042940819E-2</v>
+        <v>8.4506616525652944E-2</v>
       </c>
       <c r="J22" s="2">
-        <v>7.9562964955743665E-2</v>
+        <v>7.7678758376418688E-2</v>
       </c>
       <c r="K22" s="2">
-        <v>-6.0000000000004494E-4</v>
+        <v>-1.929999999999998E-2</v>
       </c>
       <c r="L22" s="2">
-        <v>1.454091000000002E-2</v>
+        <v>7.5547042400001541E-3</v>
       </c>
       <c r="M22" s="2">
-        <v>2.7383200000000048E-2</v>
+        <v>7.5547042400001541E-3</v>
       </c>
       <c r="N22" s="2">
-        <v>0.16857064026149021</v>
+        <v>0.11981358892363091</v>
       </c>
       <c r="O22" s="2">
-        <v>7.8351080805980189E-2</v>
+        <v>7.292593606277098E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>9.3119569427335902E-2</v>
+        <v>0.10200728456308911</v>
       </c>
       <c r="Q22" s="2">
-        <v>7.20206902255216E-2</v>
+        <v>6.8785506940236552E-2</v>
       </c>
       <c r="R22" s="2">
-        <v>7.6882374514131824E-2</v>
+        <v>7.4921977550927998E-2</v>
       </c>
       <c r="S22" s="2">
         <v>0.1847901072070588</v>
@@ -2890,7 +2890,7 @@
         <v>-1.6408690648921479E-2</v>
       </c>
       <c r="AG22">
-        <v>19726848.460000001</v>
+        <v>19490275.800000001</v>
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.25">
@@ -2901,52 +2901,52 @@
         <v>37</v>
       </c>
       <c r="C23" s="2">
-        <v>-6.7880000000000162E-3</v>
+        <v>-2.72365E-2</v>
       </c>
       <c r="D23" s="2">
-        <v>4.1896258212239079E-2</v>
+        <v>6.7889712548823136E-3</v>
       </c>
       <c r="E23" s="2">
-        <v>3.4978153739199991E-2</v>
+        <v>6.7889712548823136E-3</v>
       </c>
       <c r="F23" s="2">
-        <v>0.21055853512591319</v>
+        <v>0.15665176071501441</v>
       </c>
       <c r="G23" s="2">
-        <v>0.15860979903130759</v>
+        <v>0.13757631582783911</v>
       </c>
       <c r="H23" s="2">
-        <v>0.1456791414784904</v>
+        <v>0.1546740656270009</v>
       </c>
       <c r="I23" s="2">
-        <v>0.10452799556353611</v>
+        <v>0.1028783972688367</v>
       </c>
       <c r="J23" s="2">
-        <v>0.11463783363348901</v>
+        <v>0.1117402436729269</v>
       </c>
       <c r="K23" s="2">
-        <v>-1.2499999999999961E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L23" s="2">
-        <v>2.9880537499999971E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M23" s="2">
-        <v>2.9468749999999929E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N23" s="2">
-        <v>0.2279335112320855</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O23" s="2">
-        <v>0.1406458000440951</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P23" s="2">
-        <v>0.1663213492098834</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.12248757151155699</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R23" s="2">
-        <v>0.13418966053852779</v>
+        <v>0.12961201242848031</v>
       </c>
       <c r="S23" s="2">
         <v>0.26716999713421141</v>
@@ -2991,7 +2991,7 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG23">
-        <v>49686620.32</v>
+        <v>48140399.380000003</v>
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
@@ -3002,97 +3002,97 @@
         <v>75</v>
       </c>
       <c r="C24" s="2">
-        <v>2.3241214975864288E-3</v>
+        <v>2.233996411977746E-3</v>
       </c>
       <c r="D24" s="2">
-        <v>6.9885816688028957E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="E24" s="2">
-        <v>4.6536445359084411E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="F24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="G24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="H24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="I24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="J24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="K24" s="2">
-        <v>2.3241214975864288E-3</v>
+        <v>2.233996411977746E-3</v>
       </c>
       <c r="L24" s="2">
-        <v>6.9885816688028957E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="M24" s="2">
-        <v>4.6536445359084411E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="N24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="O24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="P24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Q24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="R24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="S24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="T24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="U24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="V24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="W24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="X24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Y24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Z24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AA24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AB24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AC24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AD24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AE24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AF24" s="2">
-        <v>2.824873600000001E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AG24">
-        <v>33829548.840000004</v>
+        <v>37358654.07</v>
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
@@ -3103,97 +3103,97 @@
         <v>76</v>
       </c>
       <c r="C25" s="2">
-        <v>2.2554219815378311E-3</v>
+        <v>2.165441593745987E-3</v>
       </c>
       <c r="D25" s="2">
-        <v>6.7815382027280879E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="E25" s="2">
-        <v>4.5159308913906848E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="F25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="G25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="H25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="I25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="J25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="K25" s="2">
-        <v>2.2554219815378311E-3</v>
+        <v>2.165441593745987E-3</v>
       </c>
       <c r="L25" s="2">
-        <v>6.7815382027280879E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="M25" s="2">
-        <v>4.5159308913906848E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="N25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="O25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="P25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Q25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="R25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="T25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="U25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="V25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="W25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="X25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Y25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Z25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AA25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AB25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AC25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AD25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AE25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AF25" s="2">
-        <v>2.7403337999999999E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AG25">
-        <v>120284577.84</v>
+        <v>130317840.72</v>
       </c>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
@@ -3204,52 +3204,52 @@
         <v>77</v>
       </c>
       <c r="C26" s="2">
-        <v>1.0799999999999921E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="D26" s="2">
-        <v>1.393457166399981E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="E26" s="2">
-        <v>1.352915999999982E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="F26" s="2">
-        <v>0.20892102861296771</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="G26" s="2">
-        <v>0.13472815943675381</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="H26" s="2">
-        <v>0.16268706625506771</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="I26" s="2">
-        <v>0.1207373590525465</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="J26" s="2">
-        <v>9.3237092723982951E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="K26" s="2">
-        <v>-1.2499999999999961E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L26" s="2">
-        <v>2.9880537499999971E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M26" s="2">
-        <v>2.9468749999999929E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N26" s="2">
-        <v>0.2279335112320855</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O26" s="2">
-        <v>0.1406458000440951</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P26" s="2">
-        <v>0.1663213492098834</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.12248757151155699</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R26" s="2">
-        <v>9.4006958248271877E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="S26" s="2">
         <v>0.29426365037508218</v>
@@ -3294,7 +3294,7 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG26">
-        <v>566421.62</v>
+        <v>-388310.68</v>
       </c>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
@@ -3305,52 +3305,52 @@
         <v>78</v>
       </c>
       <c r="C27" s="3">
-        <v>1.2999999999999901E-2</v>
+        <v>4.8999999999999044E-3</v>
       </c>
       <c r="D27" s="3">
-        <v>2.8001699340000071E-2</v>
+        <v>4.4634348939999617E-2</v>
       </c>
       <c r="E27" s="3">
-        <v>3.9540599999999808E-2</v>
+        <v>4.4634348939999617E-2</v>
       </c>
       <c r="F27" s="3">
-        <v>0.170802098022663</v>
+        <v>0.1471714394529775</v>
       </c>
       <c r="G27" s="3">
-        <v>6.4271526647182275E-2</v>
+        <v>5.9735800208212897E-2</v>
       </c>
       <c r="H27" s="3">
-        <v>6.4043482811291463E-2</v>
+        <v>9.5739784718764209E-2</v>
       </c>
       <c r="I27" s="3">
-        <v>5.2621985378944032E-2</v>
+        <v>5.4817279669409753E-2</v>
       </c>
       <c r="J27" s="3">
-        <v>6.4674870986276112E-2</v>
+        <v>6.465804985048651E-2</v>
       </c>
       <c r="K27" s="3">
-        <v>1.2999999999999901E-2</v>
+        <v>4.8999999999999044E-3</v>
       </c>
       <c r="L27" s="3">
-        <v>2.8001699340000071E-2</v>
+        <v>4.4634348939999617E-2</v>
       </c>
       <c r="M27" s="3">
-        <v>3.9540599999999808E-2</v>
+        <v>4.4634348939999617E-2</v>
       </c>
       <c r="N27" s="3">
-        <v>0.170802098022663</v>
+        <v>0.1471714394529775</v>
       </c>
       <c r="O27" s="3">
-        <v>6.4271526647182275E-2</v>
+        <v>5.9735800208212897E-2</v>
       </c>
       <c r="P27" s="3">
-        <v>6.4043482811291463E-2</v>
+        <v>9.5739784718764209E-2</v>
       </c>
       <c r="Q27" s="3">
-        <v>5.2621985378944032E-2</v>
+        <v>5.4817279669409753E-2</v>
       </c>
       <c r="R27" s="3">
-        <v>6.4674870986276112E-2</v>
+        <v>6.465804985048651E-2</v>
       </c>
       <c r="S27" s="3">
         <v>0.124788964358634</v>
@@ -3395,7 +3395,7 @@
         <v>2.0091365915979601E-2</v>
       </c>
       <c r="AG27">
-        <v>8496363.8900000006</v>
+        <v>8548924.7799999993</v>
       </c>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
@@ -3406,52 +3406,52 @@
         <v>79</v>
       </c>
       <c r="C28" s="3">
-        <v>-8.0935342777976871E-5</v>
+        <v>-4.4956476869166817E-3</v>
       </c>
       <c r="D28" s="3">
-        <v>1.041737660673658E-2</v>
+        <v>1.204120466317127E-3</v>
       </c>
       <c r="E28" s="3">
-        <v>5.7255080201208397E-3</v>
+        <v>1.204120466317127E-3</v>
       </c>
       <c r="F28" s="3">
-        <v>7.0769775235454357E-2</v>
+        <v>5.7451663866389557E-2</v>
       </c>
       <c r="G28" s="3">
-        <v>6.6794600907987611E-2</v>
+        <v>6.5058383717856438E-2</v>
       </c>
       <c r="H28" s="3">
-        <v>5.5185384468519061E-2</v>
+        <v>8.4389125465835102E-2</v>
       </c>
       <c r="I28" s="3">
-        <v>4.4717103155460507E-2</v>
+        <v>4.3810039102771807E-2</v>
       </c>
       <c r="J28" s="3">
-        <v>5.006258815824971E-2</v>
+        <v>4.9659413442706191E-2</v>
       </c>
       <c r="K28" s="3">
-        <v>-8.0935342777976871E-5</v>
+        <v>-4.4956476869166817E-3</v>
       </c>
       <c r="L28" s="3">
-        <v>1.041737660673658E-2</v>
+        <v>1.204120466317127E-3</v>
       </c>
       <c r="M28" s="3">
-        <v>5.7255080201208397E-3</v>
+        <v>1.204120466317127E-3</v>
       </c>
       <c r="N28" s="3">
-        <v>7.0769775235454357E-2</v>
+        <v>5.7451663866389557E-2</v>
       </c>
       <c r="O28" s="3">
-        <v>6.6794600907987611E-2</v>
+        <v>6.5058383717856438E-2</v>
       </c>
       <c r="P28" s="3">
-        <v>5.5185384468519061E-2</v>
+        <v>8.4389125465835102E-2</v>
       </c>
       <c r="Q28" s="3">
-        <v>4.4717103155460507E-2</v>
+        <v>4.3810039102771807E-2</v>
       </c>
       <c r="R28" s="3">
-        <v>5.006258815824971E-2</v>
+        <v>4.9659413442706191E-2</v>
       </c>
       <c r="S28" s="3">
         <v>8.0714217637701147E-2</v>
@@ -3504,52 +3504,52 @@
         <v>54</v>
       </c>
       <c r="C29" s="3">
-        <v>1.727040000000013E-3</v>
+        <v>-2.4999999999999471E-3</v>
       </c>
       <c r="D29" s="3">
-        <v>5.3565368763467847E-2</v>
+        <v>6.2756190843859638E-2</v>
       </c>
       <c r="E29" s="3">
-        <v>6.5419740194345488E-2</v>
+        <v>6.2756190843859638E-2</v>
       </c>
       <c r="F29" s="3">
-        <v>9.2357935205118924E-2</v>
+        <v>7.198561958233185E-2</v>
       </c>
       <c r="G29" s="3">
-        <v>8.6845983915933234E-2</v>
+        <v>8.9599686195299677E-2</v>
       </c>
       <c r="H29" s="3">
-        <v>9.1369689936083631E-2</v>
+        <v>0.1094516692448386</v>
       </c>
       <c r="I29" s="3">
-        <v>6.2527939087650086E-2</v>
+        <v>6.2380306064939939E-2</v>
       </c>
       <c r="J29" s="3">
-        <v>7.5988108111384678E-2</v>
+        <v>7.5085033687210423E-2</v>
       </c>
       <c r="K29" s="3">
-        <v>1.3700000000000051E-2</v>
+        <v>-3.800000000000026E-3</v>
       </c>
       <c r="L29" s="3">
-        <v>7.913111143400009E-2</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="M29" s="3">
-        <v>7.4724740000000178E-2</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="N29" s="3">
-        <v>0.16088398918518679</v>
+        <v>0.1209388679134276</v>
       </c>
       <c r="O29" s="3">
-        <v>0.1100918047856789</v>
+        <v>0.1174481059475172</v>
       </c>
       <c r="P29" s="3">
-        <v>0.1128371284909728</v>
+        <v>0.12467008367003379</v>
       </c>
       <c r="Q29" s="3">
-        <v>7.3560596447728166E-2</v>
+        <v>7.144945945259229E-2</v>
       </c>
       <c r="R29" s="3">
-        <v>7.5666529305396413E-2</v>
+        <v>7.4629602773880421E-2</v>
       </c>
       <c r="S29" s="3">
         <v>9.2049378719037733E-2</v>

</xml_diff>

<commit_message>
fix[Excel] revert the excel file
</commit_message>
<xml_diff>
--- a/app/static/returns/returns.xlsx
+++ b/app/static/returns/returns.xlsx
@@ -1,26 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneaviso-my.sharepoint.com/personal/oelassaad_aviso_ca/Documents/Development/MAP Dev/performance-scripts/performance/IPS Quarterly Returns/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work Files\ips generator\ips_generator\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1682" documentId="11_9891947AA2720024352D4C0DB503779345D63292" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14E02A51-A500-49FC-9280-8A346A7B642C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3799630-C69A-4CBE-A1E3-585352F4DA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3555" yWindow="4800" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
+  <si>
+    <t>Strategy</t>
+  </si>
   <si>
     <t>Benchmark</t>
   </si>
@@ -73,160 +92,175 @@
     <t>SIb</t>
   </si>
   <si>
+    <t>2023b</t>
+  </si>
+  <si>
+    <t>2022b</t>
+  </si>
+  <si>
+    <t>2021b</t>
+  </si>
+  <si>
+    <t>2020b</t>
+  </si>
+  <si>
+    <t>2019b</t>
+  </si>
+  <si>
+    <t>2018b</t>
+  </si>
+  <si>
+    <t>Beutel Goodman Conservative Balanced</t>
+  </si>
+  <si>
+    <t>70% FTSE Canada Universe Bond Index; 22.5% S&amp;P/TSX Composite TR Index; 7.5% S&amp;P 500 TR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Beutel Goodman Structured Bond</t>
+  </si>
+  <si>
+    <t>65% FTSE Canada Short-Term Bond Index; 35% FTSE Canada Mid-Term Bond Index</t>
+  </si>
+  <si>
+    <t>Dixon Mitchell Total Equity</t>
+  </si>
+  <si>
+    <t>70% S&amp;P/TSX 60 TR Index; 30% S&amp;P 500 TR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Balanced (RI)</t>
+  </si>
+  <si>
+    <t>60% S&amp;P/TSX Composite TR Index; 40% FTSE Canada Universe Bond Index</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Equity (RI)</t>
+  </si>
+  <si>
+    <t>S&amp;P/TSX Composite TR Index</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Bond (RI)</t>
+  </si>
+  <si>
+    <t>FTSE Canada Universe Bond Index</t>
+  </si>
+  <si>
+    <t>Guardian Global Dividend</t>
+  </si>
+  <si>
+    <t>MSCI World NR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Guardian Global Equity (RI)</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Equity Income</t>
+  </si>
+  <si>
+    <t>S&amp;P/TSX High Dividend TR Index</t>
+  </si>
+  <si>
+    <t>Jarislowsky Fraser North American Balanced</t>
+  </si>
+  <si>
+    <t>50% FTSE Canada Universe Bond Index; 25% S&amp;P/TSX Composite TR Index; 25% S&amp;P 500 TR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Jarislowsky Fraser North American Equity</t>
+  </si>
+  <si>
+    <t>50% S&amp;P/TSX Composite TR Index; 50% S&amp;P 500 TR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Manning &amp; Napier US Equity (RI)</t>
+  </si>
+  <si>
+    <t>S&amp;P 500 TR Index (CAD)</t>
+  </si>
+  <si>
+    <t>QV Dividend Income (RI)</t>
+  </si>
+  <si>
+    <t>QV Small Cap (RI)</t>
+  </si>
+  <si>
+    <t>S&amp;P TSX Small Cap Index TR</t>
+  </si>
+  <si>
+    <t>Scheer Rowlett Canadian Equity</t>
+  </si>
+  <si>
+    <t>Lazard Global Equity</t>
+  </si>
+  <si>
+    <t>MSCI All Country World NR Index</t>
+  </si>
+  <si>
+    <t>Lazard International Equity</t>
+  </si>
+  <si>
+    <t>MSCI EAFE NR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Sionna Canadian Equity</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Equity Fund</t>
+  </si>
+  <si>
+    <t>Guardian Canadian Bond Fund</t>
+  </si>
+  <si>
+    <t>Guardian Balanced Fund</t>
+  </si>
+  <si>
+    <t>40% FTSE Canada Universe Bond Index; 30% S&amp;P/TSX 60 TR Index; 30% MSCI World NR Index (CAD)</t>
+  </si>
+  <si>
+    <t>Guardian Global Dividend Fund</t>
+  </si>
+  <si>
+    <t>Brookfield Private Real Assets Fund</t>
+  </si>
+  <si>
+    <t>Aviso 5-year Bond Ladder (Taxable)</t>
+  </si>
+  <si>
+    <t>Aviso 5-year Bond Ladder (Income)</t>
+  </si>
+  <si>
+    <t>2023a</t>
+  </si>
+  <si>
+    <t>2022a</t>
+  </si>
+  <si>
+    <t>2021a</t>
+  </si>
+  <si>
+    <t>2020a</t>
+  </si>
+  <si>
+    <t>2019a</t>
+  </si>
+  <si>
+    <t>2018a</t>
+  </si>
+  <si>
+    <t>Hamilton Lane Global Private Assets Fund</t>
+  </si>
+  <si>
+    <t>2024a</t>
+  </si>
+  <si>
     <t>2024b</t>
   </si>
   <si>
-    <t>2023b</t>
-  </si>
-  <si>
-    <t>2022b</t>
-  </si>
-  <si>
-    <t>2021b</t>
-  </si>
-  <si>
-    <t>2020b</t>
-  </si>
-  <si>
-    <t>2019b</t>
-  </si>
-  <si>
-    <t>2018b</t>
-  </si>
-  <si>
-    <t>Total Market Value</t>
-  </si>
-  <si>
-    <t>Mandate</t>
-  </si>
-  <si>
-    <t>Beutel Goodman Conservative Balanced</t>
-  </si>
-  <si>
-    <t>Beutel Goodman Structured Bond</t>
-  </si>
-  <si>
-    <t>Dixon Mitchell Total Equity</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Balanced (RI)</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Equity (RI)</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Bond (RI)</t>
-  </si>
-  <si>
-    <t>Guardian Global Dividend</t>
-  </si>
-  <si>
-    <t>Guardian Global Equity (RI)</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Equity Income</t>
-  </si>
-  <si>
-    <t>Jarislowsky Fraser North American Balanced</t>
-  </si>
-  <si>
-    <t>Jarislowsky Fraser North American Equity</t>
-  </si>
-  <si>
-    <t>Manning &amp; Napier US Equity (RI)</t>
-  </si>
-  <si>
-    <t>QV Dividend Income (RI)</t>
-  </si>
-  <si>
-    <t>QV Small Cap (RI)</t>
-  </si>
-  <si>
-    <t>Scheer Rowlett Canadian Equity</t>
-  </si>
-  <si>
-    <t>Lazard Global Equity</t>
-  </si>
-  <si>
-    <t>Lazard International Equity</t>
-  </si>
-  <si>
-    <t>Sionna Canadian Equity</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Equity Fund</t>
-  </si>
-  <si>
-    <t>Guardian Canadian Bond Fund</t>
-  </si>
-  <si>
-    <t>Guardian Balanced Fund</t>
-  </si>
-  <si>
-    <t>Guardian Global Dividend Fund</t>
-  </si>
-  <si>
-    <t>Aviso 5-year Bond Ladder (Income)</t>
-  </si>
-  <si>
-    <t>Aviso 5-year Bond Ladder (Taxable)</t>
-  </si>
-  <si>
-    <t>Hamilton Lane Global Private Assets</t>
-  </si>
-  <si>
-    <t>Brookfield Private Real Assets Fund</t>
-  </si>
-  <si>
     <t>Sagard Private Credit Fund</t>
   </si>
   <si>
     <t>Mawer EAFE Large Cap Fund</t>
-  </si>
-  <si>
-    <t>70% FTSE Canada Universe Bond Index; 22.5% S&amp;P/TSX Composite TR Index; 7.5% S&amp;P 500 TR Index (CAD)</t>
-  </si>
-  <si>
-    <t>65% FTSE Canada Short-Term Bond Index; 35% FTSE Canada Mid-Term Bond Index</t>
-  </si>
-  <si>
-    <t>70% S&amp;P/TSX 60 TR Index; 30% S&amp;P 500 TR Index (CAD)</t>
-  </si>
-  <si>
-    <t>60% S&amp;P/TSX Composite TR Index; 40% FTSE Canada Universe Bond Index</t>
-  </si>
-  <si>
-    <t>S&amp;P/TSX Composite TR Index</t>
-  </si>
-  <si>
-    <t>FTSE Canada Universe Bond Index</t>
-  </si>
-  <si>
-    <t>MSCI World NR Index (CAD)</t>
-  </si>
-  <si>
-    <t>S&amp;P/TSX High Dividend TR Index</t>
-  </si>
-  <si>
-    <t>50% FTSE Canada Universe Bond Index; 25% S&amp;P/TSX Composite TR Index; 25% S&amp;P 500 TR Index (CAD)</t>
-  </si>
-  <si>
-    <t>50% S&amp;P/TSX Composite TR Index; 50% S&amp;P 500 TR Index (CAD)</t>
-  </si>
-  <si>
-    <t>S&amp;P 500 TR Index (CAD)</t>
-  </si>
-  <si>
-    <t>S&amp;P TSX Small Cap Index TR</t>
-  </si>
-  <si>
-    <t>MSCI All Country World NR Index</t>
-  </si>
-  <si>
-    <t>MSCI EAFE NR Index (CAD)</t>
-  </si>
-  <si>
-    <t>40% FTSE Canada Universe Bond Index; 30% S&amp;P/TSX 60 TR Index; 30% MSCI World NR Index (CAD)</t>
   </si>
   <si>
     <t>Aviso 5-year Bond Ladder (Income) Bench</t>
@@ -252,7 +286,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -260,14 +301,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -280,7 +314,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -288,42 +322,23 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -336,9 +351,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -346,44 +361,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -411,14 +426,31 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -446,9 +478,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -457,255 +506,252 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
+            <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6735C09-F373-4DF4-94E4-3820E8317037}">
   <dimension ref="A1:AG29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="T1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="U1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="V1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="W1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="X1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="Y1" s="1">
-        <v>2018</v>
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>18</v>
@@ -725,64 +771,61 @@
       <c r="AF1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AG1" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>26</v>
+      <c r="A2" t="s">
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2">
-        <v>6.4766065573771403E-3</v>
+        <v>-5.1765416666667008E-3</v>
       </c>
       <c r="D2" s="2">
-        <v>1.3934561058376319E-2</v>
+        <v>2.7077582276642479E-2</v>
       </c>
       <c r="E2" s="2">
-        <v>4.1389457558565823E-2</v>
+        <v>2.7077582276642479E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>0.1055936614220325</v>
+        <v>8.760456306811637E-2</v>
       </c>
       <c r="G2" s="2">
-        <v>6.6158371848539899E-2</v>
+        <v>3.9439975710667152E-2</v>
       </c>
       <c r="H2" s="2">
-        <v>5.3137582555110807E-2</v>
+        <v>6.3877404467325816E-2</v>
       </c>
       <c r="I2" s="2">
-        <v>5.0274537966843218E-2</v>
+        <v>4.6876134153442273E-2</v>
       </c>
       <c r="J2" s="2">
-        <v>6.0030081433420028E-2</v>
+        <v>6.006636732624715E-2</v>
       </c>
       <c r="K2" s="2">
-        <v>1.019999999999999E-2</v>
+        <v>-9.7000000000000419E-3</v>
       </c>
       <c r="L2" s="2">
-        <v>1.8948938120000092E-2</v>
+        <v>1.4365795256000119E-2</v>
       </c>
       <c r="M2" s="2">
-        <v>3.3586949941350593E-2</v>
+        <v>1.4365795256000119E-2</v>
       </c>
       <c r="N2" s="2">
-        <v>0.1116523111242109</v>
+        <v>0.1006594426218692</v>
       </c>
       <c r="O2" s="2">
-        <v>8.182393955332623E-2</v>
+        <v>4.5985483676901362E-2</v>
       </c>
       <c r="P2" s="2">
-        <v>4.2703236234141739E-2</v>
+        <v>5.7058368915306801E-2</v>
       </c>
       <c r="Q2" s="2">
-        <v>4.7675208314213569E-2</v>
+        <v>4.4279449003390647E-2</v>
       </c>
       <c r="R2" s="2">
-        <v>5.4269485265538993E-2</v>
+        <v>5.3996900192045949E-2</v>
       </c>
       <c r="S2" s="2">
         <v>7.110857750516808E-2</v>
@@ -827,63 +870,63 @@
         <v>-3.3133518868777578E-4</v>
       </c>
       <c r="AG2">
-        <v>38242071.369999997</v>
+        <v>36301330.950000003</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
       <c r="C3" s="2">
-        <v>2.2431480000000281E-3</v>
+        <v>1.1945763888889791E-3</v>
       </c>
       <c r="D3" s="2">
-        <v>1.940774494427089E-3</v>
+        <v>1.9544161845127968E-2</v>
       </c>
       <c r="E3" s="2">
-        <v>2.1522867150379099E-2</v>
+        <v>1.9544161845127968E-2</v>
       </c>
       <c r="F3" s="2">
-        <v>6.7164870077768279E-2</v>
+        <v>7.5732318422108147E-2</v>
       </c>
       <c r="G3" s="2">
-        <v>4.5049602682181833E-2</v>
+        <v>3.3042272690110293E-2</v>
       </c>
       <c r="H3" s="2">
-        <v>9.579391381833835E-3</v>
+        <v>1.7037497289668298E-2</v>
       </c>
       <c r="I3" s="2">
-        <v>1.8885830099319541E-2</v>
+        <v>1.786013745752291E-2</v>
       </c>
       <c r="J3" s="2">
-        <v>4.375526677979602E-2</v>
+        <v>4.4082138868742682E-2</v>
       </c>
       <c r="K3" s="2">
-        <v>2.5999999999999361E-3</v>
+        <v>2.0000000000000022E-3</v>
       </c>
       <c r="L3" s="2">
-        <v>1.9984901300000861E-3</v>
+        <v>2.0215197680000019E-2</v>
       </c>
       <c r="M3" s="2">
-        <v>2.2254087683039488E-2</v>
+        <v>2.0215197680000019E-2</v>
       </c>
       <c r="N3" s="2">
-        <v>6.6970823135683588E-2</v>
+        <v>7.6564487321105101E-2</v>
       </c>
       <c r="O3" s="2">
-        <v>4.5544669952795942E-2</v>
+        <v>3.5536843454010203E-2</v>
       </c>
       <c r="P3" s="2">
-        <v>1.221329943752991E-2</v>
+        <v>1.7954699742264161E-2</v>
       </c>
       <c r="Q3" s="2">
-        <v>1.9220883346398931E-2</v>
+        <v>1.8726063676071329E-2</v>
       </c>
       <c r="R3" s="2">
-        <v>4.1202021355724483E-2</v>
+        <v>4.1503175432556549E-2</v>
       </c>
       <c r="S3" s="2">
         <v>5.1696869975270232E-2</v>
@@ -928,63 +971,63 @@
         <v>1.9121810314036921E-2</v>
       </c>
       <c r="AG3">
-        <v>91971385.530000001</v>
+        <v>92256175.709999993</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2">
-        <v>2.062219277108435E-2</v>
+        <v>-3.7887260504201659E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>5.3552617863060759E-2</v>
+        <v>-6.7613746342441994E-3</v>
       </c>
       <c r="E4" s="2">
-        <v>4.6429153916799581E-2</v>
+        <v>-6.7613746342441994E-3</v>
       </c>
       <c r="F4" s="2">
-        <v>0.1506263396876262</v>
+        <v>0.10747436102419949</v>
       </c>
       <c r="G4" s="2">
-        <v>0.19052681859449791</v>
+        <v>0.1184281154008668</v>
       </c>
       <c r="H4" s="2">
-        <v>0.17751597544911449</v>
+        <v>0.1924759110367282</v>
       </c>
       <c r="I4" s="2">
-        <v>0.13116838095324601</v>
+        <v>0.12344629350343279</v>
       </c>
       <c r="J4" s="2">
-        <v>9.9182195825684216E-2</v>
+        <v>9.7916033221743914E-2</v>
       </c>
       <c r="K4" s="2">
-        <v>2.849999999999997E-2</v>
+        <v>-3.080000000000005E-2</v>
       </c>
       <c r="L4" s="2">
-        <v>6.8802574729999844E-2</v>
+        <v>-5.9036552800006969E-4</v>
       </c>
       <c r="M4" s="2">
-        <v>6.8171590533641524E-2</v>
+        <v>-5.9036552800006969E-4</v>
       </c>
       <c r="N4" s="2">
-        <v>0.228514766332478</v>
+        <v>0.15733752172095031</v>
       </c>
       <c r="O4" s="2">
-        <v>0.1751519605071683</v>
+        <v>9.8414974336139105E-2</v>
       </c>
       <c r="P4" s="2">
-        <v>0.15586823555346041</v>
+        <v>0.17333381896318539</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.11477365379137459</v>
+        <v>0.1056276388211768</v>
       </c>
       <c r="R4" s="2">
-        <v>6.9776228263879636E-2</v>
+        <v>6.7631197738589943E-2</v>
       </c>
       <c r="S4" s="2">
         <v>0.20300051409891351</v>
@@ -1029,63 +1072,63 @@
         <v>-4.0965727438507897E-2</v>
       </c>
       <c r="AG4">
-        <v>206259468.94999999</v>
+        <v>186211715.16999999</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>29</v>
+      <c r="A5" t="s">
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2">
-        <v>2.1507232558139581E-2</v>
+        <v>-9.0119230769231118E-3</v>
       </c>
       <c r="D5" s="2">
-        <v>6.6701393835959966E-2</v>
+        <v>2.0449601669698451E-2</v>
       </c>
       <c r="E5" s="2">
-        <v>8.8515012440417262E-2</v>
+        <v>2.0449601669698451E-2</v>
       </c>
       <c r="F5" s="2">
-        <v>0.2069181162686915</v>
+        <v>0.13595271102089471</v>
       </c>
       <c r="G5" s="2">
-        <v>0.1422469647626379</v>
+        <v>8.2214642489835565E-2</v>
       </c>
       <c r="H5" s="2">
-        <v>0.1071219142607331</v>
+        <v>0.1139290118596934</v>
       </c>
       <c r="I5" s="2">
-        <v>7.5133022668533389E-2</v>
+        <v>6.5610391484684616E-2</v>
       </c>
       <c r="J5" s="2">
-        <v>7.8989632808853294E-2</v>
+        <v>7.7280936573876025E-2</v>
       </c>
       <c r="K5" s="2">
-        <v>1.7700000000000049E-2</v>
+        <v>-1.019999999999999E-2</v>
       </c>
       <c r="L5" s="2">
-        <v>4.8325768224000143E-2</v>
+        <v>1.726833572000008E-2</v>
       </c>
       <c r="M5" s="2">
-        <v>6.6428609533619287E-2</v>
+        <v>1.726833572000008E-2</v>
       </c>
       <c r="N5" s="2">
-        <v>0.1795405094264271</v>
+        <v>0.12542782566260799</v>
       </c>
       <c r="O5" s="2">
-        <v>0.11353946446012329</v>
+        <v>5.778076241459229E-2</v>
       </c>
       <c r="P5" s="2">
-        <v>8.8070538640133256E-2</v>
+        <v>0.1035994179696009</v>
       </c>
       <c r="Q5" s="2">
-        <v>6.7143602015746984E-2</v>
+        <v>6.0336104317869843E-2</v>
       </c>
       <c r="R5" s="2">
-        <v>7.5190638967507439E-2</v>
+        <v>7.4104034579170364E-2</v>
       </c>
       <c r="S5" s="2">
         <v>0.16909176936559361</v>
@@ -1130,63 +1173,63 @@
         <v>-4.6556803672422993E-2</v>
       </c>
       <c r="AG5">
-        <v>20673836.600000001</v>
+        <v>18333995.43</v>
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>30</v>
+      <c r="A6" t="s">
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C6" s="2">
-        <v>3.1918066666666738E-2</v>
+        <v>-1.210428571428568E-2</v>
       </c>
       <c r="D6" s="2">
-        <v>0.106652512761497</v>
+        <v>1.864060358322717E-2</v>
       </c>
       <c r="E6" s="2">
-        <v>0.12728118355626639</v>
+        <v>1.864060358322717E-2</v>
       </c>
       <c r="F6" s="2">
-        <v>0.29194426639414739</v>
+        <v>0.16844499389353601</v>
       </c>
       <c r="G6" s="2">
-        <v>0.19664739335041251</v>
+        <v>0.1121131986151627</v>
       </c>
       <c r="H6" s="2">
-        <v>0.17083632575058291</v>
+        <v>0.17394038629166131</v>
       </c>
       <c r="I6" s="2">
-        <v>0.10278275857156551</v>
+        <v>8.8567757119815571E-2</v>
       </c>
       <c r="J6" s="2">
-        <v>8.7971000874423888E-2</v>
+        <v>8.4884353051230654E-2</v>
       </c>
       <c r="K6" s="2">
-        <v>2.90999999999999E-2</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L6" s="2">
-        <v>8.5231642040000111E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M6" s="2">
-        <v>0.10161627611346891</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N6" s="2">
-        <v>0.26355768014352893</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O6" s="2">
-        <v>0.16174791700777269</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P6" s="2">
-        <v>0.1506785074338641</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q6" s="2">
-        <v>9.6297839011893149E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R6" s="2">
-        <v>7.6894726818429682E-2</v>
+        <v>7.448544676534663E-2</v>
       </c>
       <c r="S6" s="2">
         <v>0.2464799745561268</v>
@@ -1231,63 +1274,63 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG6">
-        <v>28039786.23</v>
+        <v>22622943.23</v>
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>31</v>
+      <c r="A7" t="s">
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="C7" s="2">
-        <v>2.6693333333334119E-3</v>
+        <v>-3.418017543859619E-3</v>
       </c>
       <c r="D7" s="2">
-        <v>-2.6717918046893501E-3</v>
+        <v>2.198868032147927E-2</v>
       </c>
       <c r="E7" s="2">
-        <v>1.9258139340910811E-2</v>
+        <v>2.198868032147927E-2</v>
       </c>
       <c r="F7" s="2">
-        <v>7.1263011325580106E-2</v>
+        <v>8.3191615757522097E-2</v>
       </c>
       <c r="G7" s="2">
-        <v>4.8282948378003843E-2</v>
+        <v>2.8382404312901951E-2</v>
       </c>
       <c r="H7" s="2">
-        <v>-1.104035111474055E-3</v>
+        <v>1.226898501527063E-2</v>
       </c>
       <c r="I7" s="2">
-        <v>2.082094148007374E-2</v>
+        <v>1.9178763704715381E-2</v>
       </c>
       <c r="J7" s="2">
-        <v>5.196453931432532E-2</v>
+        <v>5.2481061802177598E-2</v>
       </c>
       <c r="K7" s="2">
-        <v>5.9999999999993392E-4</v>
+        <v>-2.8000000000000251E-3</v>
       </c>
       <c r="L7" s="2">
-        <v>-5.7050807799999834E-3</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="M7" s="2">
-        <v>1.444652343338104E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="N7" s="2">
-        <v>6.1163138184022081E-2</v>
+        <v>7.6447349264987974E-2</v>
       </c>
       <c r="O7" s="2">
-        <v>4.1885590908792292E-2</v>
+        <v>2.379636305646082E-2</v>
       </c>
       <c r="P7" s="2">
-        <v>-4.4831443170499918E-3</v>
+        <v>8.0919721626715457E-3</v>
       </c>
       <c r="Q7" s="2">
-        <v>1.8477013901331271E-2</v>
+        <v>1.7300619327857539E-2</v>
       </c>
       <c r="R7" s="2">
-        <v>5.0285682034808099E-2</v>
+        <v>5.0890382612324807E-2</v>
       </c>
       <c r="S7" s="2">
         <v>4.9758392035209147E-2</v>
@@ -1332,63 +1375,63 @@
         <v>1.4079379818825901E-2</v>
       </c>
       <c r="AG7">
-        <v>90742074.790000007</v>
+        <v>90357940.280000001</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>32</v>
+      <c r="A8" t="s">
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2">
-        <v>6.3962799999999209E-3</v>
+        <v>-3.1215904411764691E-2</v>
       </c>
       <c r="D8" s="2">
-        <v>1.023162808506028E-2</v>
+        <v>5.7615191611672936E-3</v>
       </c>
       <c r="E8" s="2">
-        <v>1.6052096967489549E-2</v>
+        <v>5.7615191611672936E-3</v>
       </c>
       <c r="F8" s="2">
-        <v>0.1093458078711156</v>
+        <v>0.15602004284453441</v>
       </c>
       <c r="G8" s="2">
-        <v>0.1718522843076</v>
+        <v>0.13273323400015791</v>
       </c>
       <c r="H8" s="2">
-        <v>0.13537838838819891</v>
+        <v>0.1551478095151588</v>
       </c>
       <c r="I8" s="2">
-        <v>0.1119906987604196</v>
+        <v>0.10734378244820771</v>
       </c>
       <c r="J8" s="2">
-        <v>0.10353358653112781</v>
+        <v>0.10425048159546151</v>
       </c>
       <c r="K8" s="2">
-        <v>3.5199999999999898E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L8" s="2">
-        <v>5.6813619887999822E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M8" s="2">
-        <v>3.8563366779366337E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N8" s="2">
-        <v>0.1592335772126752</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O8" s="2">
-        <v>0.20815735429916329</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P8" s="2">
-        <v>0.14860453496100429</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.1202924196785458</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R8" s="2">
-        <v>9.2978903224587128E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="S8" s="2">
         <v>0.25956354944849203</v>
@@ -1433,63 +1476,63 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG8">
-        <v>127413262.40000001</v>
+        <v>122930009.13</v>
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>33</v>
+      <c r="A9" t="s">
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2">
-        <v>4.2903829787233061E-3</v>
+        <v>-3.5942372093023311E-2</v>
       </c>
       <c r="D9" s="2">
-        <v>4.4484720197404126E-3</v>
+        <v>-6.235734338472243E-4</v>
       </c>
       <c r="E9" s="2">
-        <v>3.8221246369203321E-3</v>
+        <v>-6.235734338472243E-4</v>
       </c>
       <c r="F9" s="2">
-        <v>9.6659636385026726E-2</v>
+        <v>0.1517135575266855</v>
       </c>
       <c r="G9" s="2">
-        <v>0.17480332194648709</v>
+        <v>0.13471849448114859</v>
       </c>
       <c r="H9" s="2">
-        <v>0.13933365025535971</v>
+        <v>0.16098799855349261</v>
       </c>
       <c r="I9" s="2">
-        <v>0.1133374003936702</v>
+        <v>0.1097896375134306</v>
       </c>
       <c r="J9" s="2">
-        <v>8.7169172720092503E-2</v>
+        <v>8.820677654857545E-2</v>
       </c>
       <c r="K9" s="2">
-        <v>3.5199999999999898E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L9" s="2">
-        <v>5.6813619887999822E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M9" s="2">
-        <v>3.8563366779366337E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N9" s="2">
-        <v>0.1592335772126752</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O9" s="2">
-        <v>0.20815735429916329</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P9" s="2">
-        <v>0.14860453496100429</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q9" s="2">
-        <v>0.1202924196785458</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R9" s="2">
-        <v>9.9714367100615098E-2</v>
+        <v>9.7708296429523944E-2</v>
       </c>
       <c r="S9" s="2">
         <v>0.26275886187340619</v>
@@ -1534,63 +1577,63 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG9">
-        <v>42331667.700000003</v>
+        <v>39123712.670000002</v>
       </c>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>34</v>
+      <c r="A10" t="s">
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2">
-        <v>2.13211499999999E-2</v>
+        <v>6.3950454545453894E-3</v>
       </c>
       <c r="D10" s="2">
-        <v>6.5383764984105364E-2</v>
+        <v>5.1071890506063873E-2</v>
       </c>
       <c r="E10" s="2">
-        <v>0.1197949279763115</v>
+        <v>5.1071890506063873E-2</v>
       </c>
       <c r="F10" s="2">
-        <v>0.2211258763695492</v>
+        <v>0.13703988678249709</v>
       </c>
       <c r="G10" s="2">
-        <v>0.13681128954345281</v>
+        <v>7.7785554375998434E-2</v>
       </c>
       <c r="H10" s="2">
-        <v>0.17287649796508411</v>
+        <v>0.1716444837461153</v>
       </c>
       <c r="I10" s="2">
-        <v>8.7929416045070541E-2</v>
+        <v>7.875779031571617E-2</v>
       </c>
       <c r="J10" s="2">
-        <v>0.11476720756868961</v>
+        <v>0.1129563102030335</v>
       </c>
       <c r="K10" s="2">
-        <v>1.940000000000008E-2</v>
+        <v>4.8999999999999044E-3</v>
       </c>
       <c r="L10" s="2">
-        <v>5.2729588820000117E-2</v>
+        <v>2.9646225244000179E-2</v>
       </c>
       <c r="M10" s="2">
-        <v>8.3939047331181404E-2</v>
+        <v>2.9646225244000179E-2</v>
       </c>
       <c r="N10" s="2">
-        <v>0.2194874157261972</v>
+        <v>0.1415845117969303</v>
       </c>
       <c r="O10" s="2">
-        <v>0.1041080827295837</v>
+        <v>5.1073641533631919E-2</v>
       </c>
       <c r="P10" s="2">
-        <v>0.1691270607573041</v>
+        <v>0.1761650828228889</v>
       </c>
       <c r="Q10" s="2">
-        <v>8.890528087351246E-2</v>
+        <v>7.97362843438989E-2</v>
       </c>
       <c r="R10" s="2">
-        <v>0.1075223001682948</v>
+        <v>0.106236078843726</v>
       </c>
       <c r="S10" s="2">
         <v>0.13308185228320671</v>
@@ -1635,63 +1678,63 @@
         <v>-0.107731401591228</v>
       </c>
       <c r="AG10">
-        <v>14687161.470000001</v>
+        <v>12959685.77</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>35</v>
+      <c r="A11" t="s">
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2">
-        <v>2.182877533039651E-2</v>
+        <v>-2.793517094017095E-2</v>
       </c>
       <c r="D11" s="2">
-        <v>3.4795345796978523E-2</v>
+        <v>-6.9974686044145251E-3</v>
       </c>
       <c r="E11" s="2">
-        <v>2.7554397852769918E-2</v>
+        <v>-6.9974686044145251E-3</v>
       </c>
       <c r="F11" s="2">
-        <v>0.14679677115389159</v>
+        <v>0.11055124904926709</v>
       </c>
       <c r="G11" s="2">
-        <v>0.1398117945542541</v>
+        <v>8.8926692211731106E-2</v>
       </c>
       <c r="H11" s="2">
-        <v>9.5741230591227744E-2</v>
+        <v>0.1042701786341529</v>
       </c>
       <c r="I11" s="2">
-        <v>7.7735008897726221E-2</v>
+        <v>7.2921934057077031E-2</v>
       </c>
       <c r="J11" s="2">
-        <v>7.7765559245989158E-2</v>
+        <v>7.7175098624535421E-2</v>
       </c>
       <c r="K11" s="2">
-        <v>1.8299999999999979E-2</v>
+        <v>-1.9499999999999958E-2</v>
       </c>
       <c r="L11" s="2">
-        <v>3.1402262440000113E-2</v>
+        <v>3.343355630000211E-3</v>
       </c>
       <c r="M11" s="2">
-        <v>3.4850607000923788E-2</v>
+        <v>3.343355630000211E-3</v>
       </c>
       <c r="N11" s="2">
-        <v>0.13249649279837489</v>
+        <v>0.1162468002565875</v>
       </c>
       <c r="O11" s="2">
-        <v>0.1150348685397113</v>
+        <v>6.7799862845294712E-2</v>
       </c>
       <c r="P11" s="2">
-        <v>7.6006958773237931E-2</v>
+        <v>9.2129731790285385E-2</v>
       </c>
       <c r="Q11" s="2">
-        <v>7.081423528739661E-2</v>
+        <v>6.5838927258658142E-2</v>
       </c>
       <c r="R11" s="2">
-        <v>7.0876887207562245E-2</v>
+        <v>7.0353902482109154E-2</v>
       </c>
       <c r="S11" s="2">
         <v>0.18322548414762951</v>
@@ -1736,63 +1779,63 @@
         <v>-6.1622847520066406E-3</v>
       </c>
       <c r="AG11">
-        <v>106506674.19</v>
+        <v>103905181.66</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>36</v>
+      <c r="A12" t="s">
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2">
-        <v>3.5559540983606468E-2</v>
+        <v>-4.4305312500000027E-2</v>
       </c>
       <c r="D12" s="2">
-        <v>5.945221101696041E-2</v>
+        <v>-2.277153520861519E-2</v>
       </c>
       <c r="E12" s="2">
-        <v>3.5326857691942548E-2</v>
+        <v>-2.277153520861519E-2</v>
       </c>
       <c r="F12" s="2">
-        <v>0.19900814149791499</v>
+        <v>0.1417040383429102</v>
       </c>
       <c r="G12" s="2">
-        <v>0.20551776887071729</v>
+        <v>0.13551532035802749</v>
       </c>
       <c r="H12" s="2">
-        <v>0.15614433286782961</v>
+        <v>0.1655807769124944</v>
       </c>
       <c r="I12" s="2">
-        <v>0.11286254509671979</v>
+        <v>0.1049735988515956</v>
       </c>
       <c r="J12" s="2">
-        <v>0.10198089821845201</v>
+        <v>0.10067588666941329</v>
       </c>
       <c r="K12" s="2">
-        <v>3.6000000000000032E-2</v>
+        <v>-3.6100000000000021E-2</v>
       </c>
       <c r="L12" s="2">
-        <v>6.8678009279999896E-2</v>
+        <v>-1.363233923200002E-2</v>
       </c>
       <c r="M12" s="2">
-        <v>5.4109428127716352E-2</v>
+        <v>-1.363233923200002E-2</v>
       </c>
       <c r="N12" s="2">
-        <v>0.2057953085268982</v>
+        <v>0.15604014736937091</v>
       </c>
       <c r="O12" s="2">
-        <v>0.19208683191829001</v>
+        <v>0.1127104918208743</v>
       </c>
       <c r="P12" s="2">
-        <v>0.16022209502835061</v>
+        <v>0.1800864836126552</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.12262956661357501</v>
+        <v>0.1136342374131081</v>
       </c>
       <c r="R12" s="2">
-        <v>9.0581316052544825E-2</v>
+        <v>8.8855331373153934E-2</v>
       </c>
       <c r="S12" s="2">
         <v>0.28821327176199668</v>
@@ -1837,63 +1880,63 @@
         <v>-2.4421037083545372E-2</v>
       </c>
       <c r="AG12">
-        <v>37294625.5</v>
+        <v>36094359.75</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>37</v>
+      <c r="A13" t="s">
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2">
-        <v>3.4000089552238773E-2</v>
+        <v>-6.7599536231884083E-2</v>
       </c>
       <c r="D13" s="2">
-        <v>3.0130869593325119E-2</v>
+        <v>-6.031086254876461E-2</v>
       </c>
       <c r="E13" s="2">
-        <v>-3.1997211689957387E-2</v>
+        <v>-6.031086254876461E-2</v>
       </c>
       <c r="F13" s="2">
-        <v>9.3148302551933737E-2</v>
+        <v>8.5448334998118547E-2</v>
       </c>
       <c r="G13" s="2">
-        <v>0.16237498083958779</v>
+        <v>0.1101392932249632</v>
       </c>
       <c r="H13" s="2">
-        <v>0.1382304120776803</v>
+        <v>0.1717278808634366</v>
       </c>
       <c r="I13" s="2">
-        <v>0.1382054122022458</v>
+        <v>0.13358848677320401</v>
       </c>
       <c r="J13" s="2">
-        <v>9.6919039053080525E-2</v>
+        <v>9.662836043779599E-2</v>
       </c>
       <c r="K13" s="2">
-        <v>4.2899999999999938E-2</v>
+        <v>-5.7200000000000029E-2</v>
       </c>
       <c r="L13" s="2">
-        <v>5.1849041467999957E-2</v>
+        <v>-4.2059103400000082E-2</v>
       </c>
       <c r="M13" s="2">
-        <v>7.6092138717065438E-3</v>
+        <v>-4.2059103400000082E-2</v>
       </c>
       <c r="N13" s="2">
-        <v>0.148530491719469</v>
+        <v>0.1514001207452329</v>
       </c>
       <c r="O13" s="2">
-        <v>0.21948169477405341</v>
+        <v>0.1431775036972347</v>
       </c>
       <c r="P13" s="2">
-        <v>0.16596086144168901</v>
+        <v>0.18839266096490029</v>
       </c>
       <c r="Q13" s="2">
-        <v>0.14605505262386639</v>
+        <v>0.13895702040647101</v>
       </c>
       <c r="R13" s="2">
-        <v>7.4236826705645242E-2</v>
+        <v>7.2820767080817639E-2</v>
       </c>
       <c r="S13" s="2">
         <v>0.27366522335215349</v>
@@ -1938,63 +1981,63 @@
         <v>4.2275010225730332E-2</v>
       </c>
       <c r="AG13">
-        <v>61838278.009999998</v>
+        <v>58597796.509999998</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>38</v>
+      <c r="A14" t="s">
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C14" s="2">
-        <v>1.838815277777783E-2</v>
+        <v>-2.2661366906474578E-3</v>
       </c>
       <c r="D14" s="2">
-        <v>7.5964791497263429E-2</v>
+        <v>1.116373208500754E-2</v>
       </c>
       <c r="E14" s="2">
-        <v>8.7976574162439869E-2</v>
+        <v>1.116373208500754E-2</v>
       </c>
       <c r="F14" s="2">
-        <v>0.22689071885351719</v>
+        <v>0.13099004582773069</v>
       </c>
       <c r="G14" s="2">
-        <v>0.13347308251113371</v>
+        <v>8.2063146975251744E-2</v>
       </c>
       <c r="H14" s="2">
-        <v>0.16783535009318329</v>
+        <v>0.17067287764213049</v>
       </c>
       <c r="I14" s="2">
-        <v>9.0071223810074708E-2</v>
+        <v>7.8035810823603002E-2</v>
       </c>
       <c r="J14" s="2">
-        <v>0.1190809673611843</v>
+        <v>0.1171603222233009</v>
       </c>
       <c r="K14" s="2">
-        <v>2.90999999999999E-2</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L14" s="2">
-        <v>8.5231642040000111E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M14" s="2">
-        <v>0.10161627611346891</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N14" s="2">
-        <v>0.26355768014352893</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O14" s="2">
-        <v>0.16174791700777269</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P14" s="2">
-        <v>0.1506785074338641</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q14" s="2">
-        <v>9.6297839011893149E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R14" s="2">
-        <v>8.2932581414456807E-2</v>
+        <v>8.0382949158205319E-2</v>
       </c>
       <c r="S14" s="2">
         <v>0.19391940521041101</v>
@@ -2039,63 +2082,63 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG14">
-        <v>114083377.17</v>
+        <v>101817758.04000001</v>
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>39</v>
+      <c r="A15" t="s">
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C15" s="2">
-        <v>3.6725894736842069E-2</v>
+        <v>-9.1109999999999802E-3</v>
       </c>
       <c r="D15" s="2">
-        <v>0.13398991856030371</v>
+        <v>1.9400413770960471E-2</v>
       </c>
       <c r="E15" s="2">
-        <v>0.1559897921924713</v>
+        <v>1.9400413770960471E-2</v>
       </c>
       <c r="F15" s="2">
-        <v>0.26112494265221459</v>
+        <v>0.1241008883958441</v>
       </c>
       <c r="G15" s="2">
-        <v>0.1822130152594206</v>
+        <v>8.8651462309059736E-2</v>
       </c>
       <c r="H15" s="2">
-        <v>0.1828196570279628</v>
+        <v>0.19512163393811791</v>
       </c>
       <c r="I15" s="2">
-        <v>0.1010853331076897</v>
+        <v>8.881798785427919E-2</v>
       </c>
       <c r="J15" s="2">
-        <v>0.1159541613502926</v>
+        <v>0.1119716522842138</v>
       </c>
       <c r="K15" s="2">
-        <v>6.1800000000000077E-2</v>
+        <v>2.5600000000000071E-2</v>
       </c>
       <c r="L15" s="2">
-        <v>0.1174196323200003</v>
+        <v>8.8339527199998713E-3</v>
       </c>
       <c r="M15" s="2">
-        <v>0.1272908645203146</v>
+        <v>8.8339527199998713E-3</v>
       </c>
       <c r="N15" s="2">
-        <v>0.23084376297386311</v>
+        <v>0.1107579613550238</v>
       </c>
       <c r="O15" s="2">
-        <v>0.13767623281709371</v>
+        <v>1.877174809602411E-2</v>
       </c>
       <c r="P15" s="2">
-        <v>0.15656754876302109</v>
+        <v>0.2041523735077295</v>
       </c>
       <c r="Q15" s="2">
-        <v>8.0323443021825147E-2</v>
+        <v>6.9387845268587434E-2</v>
       </c>
       <c r="R15" s="2">
-        <v>6.602299353371599E-2</v>
+        <v>6.2345238662887333E-2</v>
       </c>
       <c r="S15" s="2">
         <v>0.1454564677544905</v>
@@ -2140,63 +2183,63 @@
         <v>-0.18167452986828991</v>
       </c>
       <c r="AG15">
-        <v>17026809.670000002</v>
+        <v>15321258.43</v>
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>40</v>
+      <c r="A16" t="s">
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C16" s="2">
-        <v>3.1941444444444363E-2</v>
+        <v>-2.0684363636363608E-2</v>
       </c>
       <c r="D16" s="2">
-        <v>7.8343682302147277E-2</v>
+        <v>-1.219021590950875E-2</v>
       </c>
       <c r="E16" s="2">
-        <v>6.5198439990229451E-2</v>
+        <v>-1.219021590950875E-2</v>
       </c>
       <c r="F16" s="2">
-        <v>0.20611206083487829</v>
+        <v>0.10316186048992</v>
       </c>
       <c r="G16" s="2">
-        <v>0.13118348815135211</v>
+        <v>6.4476624925824622E-2</v>
       </c>
       <c r="H16" s="2">
-        <v>0.16903987023430209</v>
+        <v>0.17601504224335079</v>
       </c>
       <c r="I16" s="2">
-        <v>0.1026619376818538</v>
+        <v>9.302266890190003E-2</v>
       </c>
       <c r="J16" s="2">
-        <v>9.7843246265695516E-2</v>
+        <v>9.5820830509585564E-2</v>
       </c>
       <c r="K16" s="2">
-        <v>2.90999999999999E-2</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L16" s="2">
-        <v>8.5231642040000111E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M16" s="2">
-        <v>0.10161627611346891</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N16" s="2">
-        <v>0.26355768014352893</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O16" s="2">
-        <v>0.16174791700777269</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P16" s="2">
-        <v>0.1506785074338641</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q16" s="2">
-        <v>9.6297839011893149E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R16" s="2">
-        <v>7.6894726818429682E-2</v>
+        <v>7.448544676534663E-2</v>
       </c>
       <c r="S16" s="2">
         <v>0.1789907355690501</v>
@@ -2241,63 +2284,63 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG16">
-        <v>5395028.9400000004</v>
+        <v>5275300.41</v>
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>41</v>
+      <c r="A17" t="s">
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2">
-        <v>6.1875944444444553E-2</v>
+        <v>-5.0939892857142843E-2</v>
       </c>
       <c r="D17" s="2">
-        <v>4.8577890096726861E-2</v>
+        <v>-2.8692617988143269E-2</v>
       </c>
       <c r="E17" s="2">
-        <v>1.8491445265368171E-2</v>
+        <v>-2.8692617988143269E-2</v>
       </c>
       <c r="F17" s="2">
-        <v>8.8455213319080128E-2</v>
+        <v>6.7028259489456454E-2</v>
       </c>
       <c r="G17" s="2">
-        <v>0.1465309131720445</v>
+        <v>9.088803846271909E-2</v>
       </c>
       <c r="H17" s="2">
-        <v>0.1059402634570261</v>
+        <v>0.1224068762633332</v>
       </c>
       <c r="I17" s="2">
-        <v>0.10264265510830969</v>
+        <v>9.5909508957356282E-2</v>
       </c>
       <c r="J17" s="2">
-        <v>8.1265799183142473E-2</v>
+        <v>7.9910729147968595E-2</v>
       </c>
       <c r="K17" s="2">
-        <v>3.6999999999999922E-2</v>
+        <v>-4.0399999999999991E-2</v>
       </c>
       <c r="L17" s="2">
-        <v>5.7380803939999891E-2</v>
+        <v>-1.25342139839999E-2</v>
       </c>
       <c r="M17" s="2">
-        <v>4.4127366680842162E-2</v>
+        <v>-1.25342139839999E-2</v>
       </c>
       <c r="N17" s="2">
-        <v>0.15861705826427741</v>
+        <v>0.1397493629826794</v>
       </c>
       <c r="O17" s="2">
-        <v>0.19628148817845359</v>
+        <v>0.12140449706502079</v>
       </c>
       <c r="P17" s="2">
-        <v>0.13725172993394569</v>
+        <v>0.15465495678796759</v>
       </c>
       <c r="Q17" s="2">
-        <v>0.1080047898544072</v>
+        <v>0.1006417652541247</v>
       </c>
       <c r="R17" s="2">
-        <v>8.1977593387603021E-2</v>
+        <v>8.0223669909337936E-2</v>
       </c>
       <c r="S17" s="2">
         <v>0.19251440061512121</v>
@@ -2342,63 +2385,63 @@
         <v>-1.2569244036318761E-2</v>
       </c>
       <c r="AG17">
-        <v>29608278.829999998</v>
+        <v>27474507.350000001</v>
       </c>
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>42</v>
+      <c r="A18" t="s">
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C18" s="2">
-        <v>2.0326516129032249E-2</v>
+        <v>-2.9110799999999989E-2</v>
       </c>
       <c r="D18" s="2">
-        <v>5.1141353967351089E-2</v>
+        <v>4.6301933509756532E-2</v>
       </c>
       <c r="E18" s="2">
-        <v>9.9811231048102522E-2</v>
+        <v>4.6301933509756532E-2</v>
       </c>
       <c r="F18" s="2">
-        <v>0.14672598451192179</v>
+        <v>7.6880360798713854E-2</v>
       </c>
       <c r="G18" s="2">
-        <v>0.15347146597702979</v>
+        <v>9.8296011522881477E-2</v>
       </c>
       <c r="H18" s="2">
-        <v>8.8004662767776409E-2</v>
+        <v>0.10389964249085031</v>
       </c>
       <c r="I18" s="2">
-        <v>6.1452052059663982E-2</v>
+        <v>5.8994578820060761E-2</v>
       </c>
       <c r="J18" s="2">
-        <v>6.72899287432982E-2</v>
+        <v>6.4242663443119241E-2</v>
       </c>
       <c r="K18" s="2">
-        <v>1.459999999999995E-2</v>
+        <v>-3.800000000000026E-3</v>
       </c>
       <c r="L18" s="2">
-        <v>6.2589849487999727E-2</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="M18" s="2">
-        <v>0.1376520316387031</v>
+        <v>7.0640785988000054E-2</v>
       </c>
       <c r="N18" s="2">
-        <v>0.17997363392522231</v>
+        <v>0.1209388679134276</v>
       </c>
       <c r="O18" s="2">
-        <v>0.1876408791383288</v>
+        <v>0.1174481059475172</v>
       </c>
       <c r="P18" s="2">
-        <v>0.11667047914568179</v>
+        <v>0.12467008367003379</v>
       </c>
       <c r="Q18" s="2">
-        <v>7.731190454466641E-2</v>
+        <v>7.144945945259229E-2</v>
       </c>
       <c r="R18" s="2">
-        <v>7.906640607421922E-2</v>
+        <v>7.524501681840956E-2</v>
       </c>
       <c r="S18" s="2">
         <v>0.1238325144064758</v>
@@ -2443,63 +2486,63 @@
         <v>-5.5537819245731417E-2</v>
       </c>
       <c r="AG18">
-        <v>21648852.649999999</v>
+        <v>18788911.550000001</v>
       </c>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>43</v>
+      <c r="A19" t="s">
+        <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C19" s="2">
-        <v>2.6215333333333261E-2</v>
+        <v>3.9472499999999577E-3</v>
       </c>
       <c r="D19" s="2">
-        <v>5.9849421237785361E-2</v>
+        <v>3.2863056265764801E-2</v>
       </c>
       <c r="E19" s="2">
-        <v>9.4679312401161342E-2</v>
+        <v>3.2863056265764801E-2</v>
       </c>
       <c r="F19" s="2">
-        <v>0.22391761076657279</v>
+        <v>0.15054358655904451</v>
       </c>
       <c r="G19" s="2">
-        <v>0.1524105865072998</v>
+        <v>9.1249189552183418E-2</v>
       </c>
       <c r="H19" s="2">
-        <v>0.16876918459595111</v>
+        <v>0.1819130928844486</v>
       </c>
       <c r="I19" s="2">
-        <v>9.7730598979577143E-2</v>
+        <v>8.8295704973029299E-2</v>
       </c>
       <c r="J19" s="2">
-        <v>8.8247180101207467E-2</v>
+        <v>8.6261410546911721E-2</v>
       </c>
       <c r="K19" s="2">
-        <v>2.90999999999999E-2</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L19" s="2">
-        <v>8.5231642040000111E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M19" s="2">
-        <v>0.10161627611346891</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N19" s="2">
-        <v>0.26355768014352893</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O19" s="2">
-        <v>0.16174791700777269</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P19" s="2">
-        <v>0.1506785074338641</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q19" s="2">
-        <v>9.6297839011893149E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R19" s="2">
-        <v>8.4317751946220154E-2</v>
+        <v>8.1026660239410964E-2</v>
       </c>
       <c r="S19" s="2">
         <v>0.17063771874488459</v>
@@ -2544,63 +2587,63 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG19">
-        <v>1254823</v>
+        <v>4214482.78</v>
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>44</v>
+      <c r="A20" t="s">
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C20" s="2">
-        <v>2.3340399999999931E-2</v>
+        <v>-2.1749600000000039E-2</v>
       </c>
       <c r="D20" s="2">
-        <v>7.131055708284495E-2</v>
+        <v>9.9861952172015656E-3</v>
       </c>
       <c r="E20" s="2">
-        <v>8.2008873444123331E-2</v>
+        <v>9.9861952172015656E-3</v>
       </c>
       <c r="F20" s="2">
-        <v>0.2013196150566037</v>
+        <v>0.1318423593638387</v>
       </c>
       <c r="G20" s="2">
-        <v>0.1703263907887673</v>
+        <v>9.8240397167722815E-2</v>
       </c>
       <c r="H20" s="2">
-        <v>0.15462179004768781</v>
+        <v>0.16899659813090301</v>
       </c>
       <c r="I20" s="2">
-        <v>9.772981062475794E-2</v>
+        <v>8.7613179492281423E-2</v>
       </c>
       <c r="J20" s="2">
-        <v>8.6523938981074577E-2</v>
+        <v>8.2816539945535839E-2</v>
       </c>
       <c r="K20" s="2">
-        <v>2.90999999999999E-2</v>
+        <v>-1.5100000000000001E-2</v>
       </c>
       <c r="L20" s="2">
-        <v>8.5231642040000111E-2</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="M20" s="2">
-        <v>0.10161627611346891</v>
+        <v>1.509782191999998E-2</v>
       </c>
       <c r="N20" s="2">
-        <v>0.26355768014352893</v>
+        <v>0.1581126941027475</v>
       </c>
       <c r="O20" s="2">
-        <v>0.16174791700777269</v>
+        <v>7.843590474826434E-2</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1506785074338641</v>
+        <v>0.16805800402612331</v>
       </c>
       <c r="Q20" s="2">
-        <v>9.6297839011893149E-2</v>
+        <v>8.5576481212968236E-2</v>
       </c>
       <c r="R20" s="2">
-        <v>7.9178860213287017E-2</v>
+        <v>7.4381651558945938E-2</v>
       </c>
       <c r="S20" s="2">
         <v>0.21693517822200331</v>
@@ -2645,63 +2688,63 @@
         <v>-8.8861093780151279E-2</v>
       </c>
       <c r="AG20">
-        <v>13267037.25</v>
+        <v>11633336.32</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>45</v>
+      <c r="A21" t="s">
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="C21" s="2">
-        <v>3.2385999999999799E-3</v>
+        <v>-2.1986999999999979E-3</v>
       </c>
       <c r="D21" s="2">
-        <v>-5.9147547327208514E-3</v>
+        <v>2.366803950823115E-2</v>
       </c>
       <c r="E21" s="2">
-        <v>1.7613294126814779E-2</v>
+        <v>2.366803950823115E-2</v>
       </c>
       <c r="F21" s="2">
-        <v>6.9503628434784304E-2</v>
+        <v>8.4854635602114037E-2</v>
       </c>
       <c r="G21" s="2">
-        <v>4.8406436900457761E-2</v>
+        <v>3.029970404733762E-2</v>
       </c>
       <c r="H21" s="2">
-        <v>-3.3333633263105118E-3</v>
+        <v>1.0661860433113681E-2</v>
       </c>
       <c r="I21" s="2">
-        <v>2.393077278735856E-2</v>
+        <v>2.2844225768598129E-2</v>
       </c>
       <c r="J21" s="2">
-        <v>2.7260611075226041E-2</v>
+        <v>2.8184191500508989E-2</v>
       </c>
       <c r="K21" s="2">
-        <v>5.9999999999993392E-4</v>
+        <v>-2.8000000000000251E-3</v>
       </c>
       <c r="L21" s="2">
-        <v>-5.7050807799999834E-3</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="M21" s="2">
-        <v>1.444652343338104E-2</v>
+        <v>2.0267230399999999E-2</v>
       </c>
       <c r="N21" s="2">
-        <v>6.1163138184022081E-2</v>
+        <v>7.6447349264987974E-2</v>
       </c>
       <c r="O21" s="2">
-        <v>4.1885590908792292E-2</v>
+        <v>2.379636305646082E-2</v>
       </c>
       <c r="P21" s="2">
-        <v>-4.4831443170499918E-3</v>
+        <v>8.0919721626715457E-3</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.8477013901331271E-2</v>
+        <v>1.7300619327857539E-2</v>
       </c>
       <c r="R21" s="2">
-        <v>2.8914800343172949E-2</v>
+        <v>2.985386050536731E-2</v>
       </c>
       <c r="S21" s="2">
         <v>4.7779083879743611E-2</v>
@@ -2746,63 +2789,63 @@
         <v>1.4079379818825901E-2</v>
       </c>
       <c r="AG21">
-        <v>14716363.48</v>
+        <v>14289819.52</v>
       </c>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>46</v>
+      <c r="A22" t="s">
+        <v>58</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C22" s="2">
-        <v>1.6798000000000091E-2</v>
+        <v>-1.805699999999999E-2</v>
       </c>
       <c r="D22" s="2">
-        <v>3.8275714925727122E-2</v>
+        <v>3.0886347110097301E-3</v>
       </c>
       <c r="E22" s="2">
-        <v>4.1482569338445067E-2</v>
+        <v>3.0886347110097301E-3</v>
       </c>
       <c r="F22" s="2">
-        <v>0.14359199128325881</v>
+        <v>0.1247030961510633</v>
       </c>
       <c r="G22" s="2">
-        <v>0.13748700862666219</v>
+        <v>8.6284729443472763E-2</v>
       </c>
       <c r="H22" s="2">
-        <v>0.12637888343476081</v>
+        <v>0.1396859127128007</v>
       </c>
       <c r="I22" s="2">
-        <v>9.0628482559299783E-2</v>
+        <v>8.4506616525652944E-2</v>
       </c>
       <c r="J22" s="2">
-        <v>7.9097642171012561E-2</v>
+        <v>7.7678758376418688E-2</v>
       </c>
       <c r="K22" s="2">
-        <v>1.9500000000000069E-2</v>
+        <v>-1.929999999999998E-2</v>
       </c>
       <c r="L22" s="2">
-        <v>4.0084520600000013E-2</v>
+        <v>7.5547042400001541E-3</v>
       </c>
       <c r="M22" s="2">
-        <v>4.7942051537735342E-2</v>
+        <v>7.5547042400001541E-3</v>
       </c>
       <c r="N22" s="2">
-        <v>0.14962856807481659</v>
+        <v>0.11981358892363091</v>
       </c>
       <c r="O22" s="2">
-        <v>0.1261733099692515</v>
+        <v>7.292593606277098E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>8.7498464844649515E-2</v>
+        <v>0.10200728456308911</v>
       </c>
       <c r="Q22" s="2">
-        <v>7.4596100789319442E-2</v>
+        <v>6.8785506940236552E-2</v>
       </c>
       <c r="R22" s="2">
-        <v>7.6516039703509842E-2</v>
+        <v>7.4921977550927998E-2</v>
       </c>
       <c r="S22" s="2">
         <v>0.1847901072070588</v>
@@ -2847,63 +2890,63 @@
         <v>-1.6408690648921479E-2</v>
       </c>
       <c r="AG22">
-        <v>19551701.530000001</v>
+        <v>19490275.800000001</v>
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>47</v>
+      <c r="A23" t="s">
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="C23" s="2">
-        <v>5.5673000000000528E-3</v>
+        <v>-2.72365E-2</v>
       </c>
       <c r="D23" s="2">
-        <v>1.34055746947872E-2</v>
+        <v>6.7889712548823136E-3</v>
       </c>
       <c r="E23" s="2">
-        <v>2.028555601092763E-2</v>
+        <v>6.7889712548823136E-3</v>
       </c>
       <c r="F23" s="2">
-        <v>0.1117676525635318</v>
+        <v>0.15665176071501441</v>
       </c>
       <c r="G23" s="2">
-        <v>0.17749429681225259</v>
+        <v>0.13757631582783911</v>
       </c>
       <c r="H23" s="2">
-        <v>0.13893451706079959</v>
+        <v>0.1546740656270009</v>
       </c>
       <c r="I23" s="2">
-        <v>0.107134023126658</v>
+        <v>0.1028783972688367</v>
       </c>
       <c r="J23" s="2">
-        <v>0.1107195820167468</v>
+        <v>0.1117402436729269</v>
       </c>
       <c r="K23" s="2">
-        <v>3.5199999999999898E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L23" s="2">
-        <v>5.6813619887999822E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M23" s="2">
-        <v>3.8563366779366337E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N23" s="2">
-        <v>0.1592335772126752</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O23" s="2">
-        <v>0.20815735429916329</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P23" s="2">
-        <v>0.14860453496100429</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.1202924196785458</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R23" s="2">
-        <v>0.13156739100778189</v>
+        <v>0.12961201242848031</v>
       </c>
       <c r="S23" s="2">
         <v>0.26716999713421141</v>
@@ -2948,265 +2991,265 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG23">
-        <v>50407811.329999998</v>
+        <v>48140399.380000003</v>
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>48</v>
+      <c r="A24" t="s">
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C24" s="2">
-        <v>2.4612767695433302E-3</v>
+        <v>2.233996411977746E-3</v>
       </c>
       <c r="D24" s="2">
-        <v>7.4020188687664579E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="E24" s="2">
-        <v>1.4858827620866769E-2</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="F24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="G24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="H24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="I24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="J24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="K24" s="2">
-        <v>2.4612767695433302E-3</v>
+        <v>2.233996411977746E-3</v>
       </c>
       <c r="L24" s="2">
-        <v>7.4020188687664579E-3</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="M24" s="2">
-        <v>1.4858827620866769E-2</v>
+        <v>6.7169726051348189E-3</v>
       </c>
       <c r="N24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="O24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="P24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Q24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="R24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="S24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="T24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="U24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="V24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="W24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="X24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Y24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="Z24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AA24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AB24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AC24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AD24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AE24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AF24" s="2">
-        <v>2.993844E-2</v>
+        <v>2.7139811E-2</v>
       </c>
       <c r="AG24">
-        <v>48648376.960000001</v>
+        <v>37358654.07</v>
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>49</v>
+      <c r="A25" t="s">
+        <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2">
-        <v>2.3551441116920202E-3</v>
+        <v>2.165441593745987E-3</v>
       </c>
       <c r="D25" s="2">
-        <v>7.0820855097233348E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="E25" s="2">
-        <v>1.4214326954613551E-2</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="F25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="G25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="H25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="I25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="J25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="K25" s="2">
-        <v>2.3551441116920202E-3</v>
+        <v>2.165441593745987E-3</v>
       </c>
       <c r="L25" s="2">
-        <v>7.0820855097233348E-3</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="M25" s="2">
-        <v>1.4214326954613551E-2</v>
+        <v>6.510402347178923E-3</v>
       </c>
       <c r="N25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="O25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="P25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Q25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="R25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="T25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="U25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="V25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="W25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="X25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Y25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="Z25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AA25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AB25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AC25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AD25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AE25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AF25" s="2">
-        <v>2.8630701000000008E-2</v>
+        <v>2.6297027000000001E-2</v>
       </c>
       <c r="AG25">
-        <v>147402558.13999999</v>
+        <v>130317840.72</v>
       </c>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>50</v>
+      <c r="A26" t="s">
+        <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C26" s="2">
-        <v>1.7611999999999961E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="D26" s="2">
-        <v>3.8858405488279901E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="E26" s="2">
-        <v>2.0918223333737052E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="F26" s="2">
-        <v>0.13953825248700241</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="G26" s="2">
-        <v>0.20127605577475821</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="H26" s="2">
-        <v>0.14467478939725781</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="I26" s="2">
-        <v>0.118374337323343</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="J26" s="2">
-        <v>9.2146810365936194E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="K26" s="2">
-        <v>3.5199999999999898E-2</v>
+        <v>-4.5400000000000003E-2</v>
       </c>
       <c r="L26" s="2">
-        <v>5.6813619887999822E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="M26" s="2">
-        <v>3.8563366779366337E-2</v>
+        <v>-1.7269131250000069E-2</v>
       </c>
       <c r="N26" s="2">
-        <v>0.1592335772126752</v>
+        <v>0.13826503187235281</v>
       </c>
       <c r="O26" s="2">
-        <v>0.20815735429916329</v>
+        <v>0.1310029398606134</v>
       </c>
       <c r="P26" s="2">
-        <v>0.14860453496100429</v>
+        <v>0.16693981620699511</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.1202924196785458</v>
+        <v>0.1130616156815176</v>
       </c>
       <c r="R26" s="2">
-        <v>9.2978903224587128E-2</v>
+        <v>9.1357505693961727E-2</v>
       </c>
       <c r="S26" s="2">
         <v>0.29426365037508218</v>
@@ -3251,310 +3294,304 @@
         <v>6.3113667818059938E-4</v>
       </c>
       <c r="AG26">
-        <v>653656.46</v>
+        <v>-388310.68</v>
       </c>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>51</v>
+      <c r="A27" t="s">
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="2">
-        <v>9.300000000000086E-3</v>
-      </c>
-      <c r="D27" s="2">
-        <v>-2.3638354104999929E-2</v>
-      </c>
-      <c r="E27" s="2">
-        <v>1.9940912289510001E-2</v>
-      </c>
-      <c r="F27" s="2">
-        <v>0.1126511403928179</v>
-      </c>
-      <c r="G27" s="2">
-        <v>8.0205572124735225E-2</v>
-      </c>
-      <c r="H27" s="2">
-        <v>7.319053656714436E-2</v>
-      </c>
-      <c r="I27" s="2">
-        <v>5.394499691859167E-2</v>
-      </c>
-      <c r="J27" s="2">
-        <v>6.2691999553548872E-2</v>
-      </c>
-      <c r="K27" s="2">
-        <v>9.300000000000086E-3</v>
-      </c>
-      <c r="L27" s="2">
-        <v>-2.3638354104999929E-2</v>
-      </c>
-      <c r="M27" s="2">
-        <v>1.9940912289510001E-2</v>
-      </c>
-      <c r="N27" s="2">
-        <v>0.1126511403928179</v>
-      </c>
-      <c r="O27" s="2">
-        <v>8.0205572124735225E-2</v>
-      </c>
-      <c r="P27" s="2">
-        <v>7.319053656714436E-2</v>
-      </c>
-      <c r="Q27" s="2">
-        <v>5.394499691859167E-2</v>
-      </c>
-      <c r="R27" s="2">
-        <v>6.2691999553548872E-2</v>
-      </c>
-      <c r="S27" s="2">
+        <v>78</v>
+      </c>
+      <c r="C27" s="3">
+        <v>4.8999999999999044E-3</v>
+      </c>
+      <c r="D27" s="3">
+        <v>4.4634348939999617E-2</v>
+      </c>
+      <c r="E27" s="3">
+        <v>4.4634348939999617E-2</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0.1471714394529775</v>
+      </c>
+      <c r="G27" s="3">
+        <v>5.9735800208212897E-2</v>
+      </c>
+      <c r="H27" s="3">
+        <v>9.5739784718764209E-2</v>
+      </c>
+      <c r="I27" s="3">
+        <v>5.4817279669409753E-2</v>
+      </c>
+      <c r="J27" s="3">
+        <v>6.465804985048651E-2</v>
+      </c>
+      <c r="K27" s="3">
+        <v>4.8999999999999044E-3</v>
+      </c>
+      <c r="L27" s="3">
+        <v>4.4634348939999617E-2</v>
+      </c>
+      <c r="M27" s="3">
+        <v>4.4634348939999617E-2</v>
+      </c>
+      <c r="N27" s="3">
+        <v>0.1471714394529775</v>
+      </c>
+      <c r="O27" s="3">
+        <v>5.9735800208212897E-2</v>
+      </c>
+      <c r="P27" s="3">
+        <v>9.5739784718764209E-2</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>5.4817279669409753E-2</v>
+      </c>
+      <c r="R27" s="3">
+        <v>6.465804985048651E-2</v>
+      </c>
+      <c r="S27" s="3">
         <v>0.124788964358634</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="3">
         <v>5.4098630863060437E-2</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="3">
         <v>-3.4202652847085679E-2</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="3">
         <v>0.1455653061407236</v>
       </c>
-      <c r="W27" s="2">
+      <c r="W27" s="3">
         <v>-8.3092281574879134E-3</v>
       </c>
-      <c r="X27" s="2">
+      <c r="X27" s="3">
         <v>0.115914764648821</v>
       </c>
-      <c r="Y27" s="2">
+      <c r="Y27" s="3">
         <v>2.0091365915979601E-2</v>
       </c>
-      <c r="Z27" s="2">
+      <c r="Z27" s="3">
         <v>0.124788964358634</v>
       </c>
-      <c r="AA27" s="2">
+      <c r="AA27" s="3">
         <v>5.4098630863060437E-2</v>
       </c>
-      <c r="AB27" s="2">
+      <c r="AB27" s="3">
         <v>-3.4202652847085679E-2</v>
       </c>
-      <c r="AC27" s="2">
+      <c r="AC27" s="3">
         <v>0.1455653061407236</v>
       </c>
-      <c r="AD27" s="2">
+      <c r="AD27" s="3">
         <v>-8.3092281574879134E-3</v>
       </c>
-      <c r="AE27" s="2">
+      <c r="AE27" s="3">
         <v>0.115914764648821</v>
       </c>
-      <c r="AF27" s="2">
+      <c r="AF27" s="3">
         <v>2.0091365915979601E-2</v>
       </c>
       <c r="AG27">
-        <v>8618778.7699999996</v>
+        <v>8548924.7799999993</v>
       </c>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>52</v>
+      <c r="A28" t="s">
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="2">
-        <v>6.506600000000029E-3</v>
-      </c>
-      <c r="D28" s="2">
-        <v>1.876838765919087E-2</v>
-      </c>
-      <c r="E28" s="2">
-        <v>1.9995107525208281E-2</v>
-      </c>
-      <c r="F28" s="2">
-        <v>5.9071636193494648E-2</v>
-      </c>
-      <c r="G28" s="2">
-        <v>8.8080506616657894E-2</v>
-      </c>
-      <c r="H28" s="2">
-        <v>6.8760021177610042E-2</v>
-      </c>
-      <c r="I28" s="2">
-        <v>4.4932211428522877E-2</v>
-      </c>
-      <c r="J28" s="2">
-        <v>4.996055002208144E-2</v>
-      </c>
-      <c r="K28" s="2">
-        <v>6.506600000000029E-3</v>
-      </c>
-      <c r="L28" s="2">
-        <v>1.876838765919087E-2</v>
-      </c>
-      <c r="M28" s="2">
-        <v>1.9995107525208281E-2</v>
-      </c>
-      <c r="N28" s="2">
-        <v>5.9071636193494648E-2</v>
-      </c>
-      <c r="O28" s="2">
-        <v>8.8080506616657894E-2</v>
-      </c>
-      <c r="P28" s="2">
-        <v>6.8760021177610042E-2</v>
-      </c>
-      <c r="Q28" s="2">
-        <v>4.4932211428522877E-2</v>
-      </c>
-      <c r="R28" s="2">
-        <v>4.996055002208144E-2</v>
-      </c>
-      <c r="S28" s="2">
+        <v>79</v>
+      </c>
+      <c r="C28" s="3">
+        <v>-4.4956476869166817E-3</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1.204120466317127E-3</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1.204120466317127E-3</v>
+      </c>
+      <c r="F28" s="3">
+        <v>5.7451663866389557E-2</v>
+      </c>
+      <c r="G28" s="3">
+        <v>6.5058383717856438E-2</v>
+      </c>
+      <c r="H28" s="3">
+        <v>8.4389125465835102E-2</v>
+      </c>
+      <c r="I28" s="3">
+        <v>4.3810039102771807E-2</v>
+      </c>
+      <c r="J28" s="3">
+        <v>4.9659413442706191E-2</v>
+      </c>
+      <c r="K28" s="3">
+        <v>-4.4956476869166817E-3</v>
+      </c>
+      <c r="L28" s="3">
+        <v>1.204120466317127E-3</v>
+      </c>
+      <c r="M28" s="3">
+        <v>1.204120466317127E-3</v>
+      </c>
+      <c r="N28" s="3">
+        <v>5.7451663866389557E-2</v>
+      </c>
+      <c r="O28" s="3">
+        <v>6.5058383717856438E-2</v>
+      </c>
+      <c r="P28" s="3">
+        <v>8.4389125465835102E-2</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>4.3810039102771807E-2</v>
+      </c>
+      <c r="R28" s="3">
+        <v>4.9659413442706191E-2</v>
+      </c>
+      <c r="S28" s="3">
         <v>8.0714217637701147E-2</v>
       </c>
-      <c r="T28" s="2">
+      <c r="T28" s="3">
         <v>0.1259456759958231</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="3">
         <v>-9.3833560932529148E-3</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="3">
         <v>5.1052418973622782E-2</v>
       </c>
-      <c r="W28" s="2">
+      <c r="W28" s="3">
         <v>1.828699955803148E-2</v>
       </c>
-      <c r="X28" s="2">
+      <c r="X28" s="3">
         <v>7.7349186294291661E-2</v>
       </c>
-      <c r="Y28" s="2">
+      <c r="Y28" s="3">
         <v>-4.6128794597813938E-3</v>
       </c>
-      <c r="Z28" s="2">
+      <c r="Z28" s="3">
         <v>8.0714217637701147E-2</v>
       </c>
-      <c r="AA28" s="2">
+      <c r="AA28" s="3">
         <v>0.1259456759958231</v>
       </c>
-      <c r="AB28" s="2">
+      <c r="AB28" s="3">
         <v>-9.3833560932529148E-3</v>
       </c>
-      <c r="AC28" s="2">
+      <c r="AC28" s="3">
         <v>5.1052418973622782E-2</v>
       </c>
-      <c r="AD28" s="2">
+      <c r="AD28" s="3">
         <v>1.828699955803148E-2</v>
       </c>
-      <c r="AE28" s="2">
+      <c r="AE28" s="3">
         <v>7.7349186294291661E-2</v>
       </c>
-      <c r="AF28" s="2">
+      <c r="AF28" s="3">
         <v>-4.6128794597813938E-3</v>
-      </c>
-      <c r="AG28">
-        <v>-95656.27</v>
       </c>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>53</v>
+      <c r="A29" t="s">
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="2">
-        <v>-1.3900000000000019E-3</v>
-      </c>
-      <c r="D29" s="2">
-        <v>6.2410980091998081E-3</v>
-      </c>
-      <c r="E29" s="2">
-        <v>6.9388956390800116E-2</v>
-      </c>
-      <c r="F29" s="2">
-        <v>0.10980135631350579</v>
-      </c>
-      <c r="G29" s="2">
-        <v>0.15027340136031531</v>
-      </c>
-      <c r="H29" s="2">
-        <v>8.8299249847922479E-2</v>
-      </c>
-      <c r="I29" s="2">
-        <v>6.3914755822128022E-2</v>
-      </c>
-      <c r="J29" s="2">
-        <v>7.3869519949001816E-2</v>
-      </c>
-      <c r="K29" s="2">
-        <v>1.459999999999995E-2</v>
-      </c>
-      <c r="L29" s="2">
-        <v>6.2589849487999727E-2</v>
-      </c>
-      <c r="M29" s="2">
-        <v>0.1376520316387031</v>
-      </c>
-      <c r="N29" s="2">
-        <v>0.17997363392522231</v>
-      </c>
-      <c r="O29" s="2">
-        <v>0.1876408791383288</v>
-      </c>
-      <c r="P29" s="2">
-        <v>0.11667047914568179</v>
-      </c>
-      <c r="Q29" s="2">
-        <v>7.731190454466641E-2</v>
-      </c>
-      <c r="R29" s="2">
-        <v>7.901022020326276E-2</v>
-      </c>
-      <c r="S29" s="2">
+        <v>54</v>
+      </c>
+      <c r="C29" s="3">
+        <v>-2.4999999999999471E-3</v>
+      </c>
+      <c r="D29" s="3">
+        <v>6.2756190843859638E-2</v>
+      </c>
+      <c r="E29" s="3">
+        <v>6.2756190843859638E-2</v>
+      </c>
+      <c r="F29" s="3">
+        <v>7.198561958233185E-2</v>
+      </c>
+      <c r="G29" s="3">
+        <v>8.9599686195299677E-2</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0.1094516692448386</v>
+      </c>
+      <c r="I29" s="3">
+        <v>6.2380306064939939E-2</v>
+      </c>
+      <c r="J29" s="3">
+        <v>7.5085033687210423E-2</v>
+      </c>
+      <c r="K29" s="3">
+        <v>-3.800000000000026E-3</v>
+      </c>
+      <c r="L29" s="3">
+        <v>7.0640785988000054E-2</v>
+      </c>
+      <c r="M29" s="3">
+        <v>7.0640785988000054E-2</v>
+      </c>
+      <c r="N29" s="3">
+        <v>0.1209388679134276</v>
+      </c>
+      <c r="O29" s="3">
+        <v>0.1174481059475172</v>
+      </c>
+      <c r="P29" s="3">
+        <v>0.12467008367003379</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>7.144945945259229E-2</v>
+      </c>
+      <c r="R29" s="3">
+        <v>7.4629602773880421E-2</v>
+      </c>
+      <c r="S29" s="3">
         <v>9.2049378719037733E-2</v>
       </c>
-      <c r="T29" s="2">
+      <c r="T29" s="3">
         <v>0.1898117381043074</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="3">
         <v>-0.1603738713607461</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="3">
         <v>0.16507135840840581</v>
       </c>
-      <c r="W29" s="2">
+      <c r="W29" s="3">
         <v>5.4079106591117247E-2</v>
       </c>
-      <c r="X29" s="2">
+      <c r="X29" s="3">
         <v>0.15845914942998779</v>
       </c>
-      <c r="Y29" s="2">
+      <c r="Y29" s="3">
         <v>-6.0255804356564857E-2</v>
       </c>
-      <c r="Z29" s="2">
+      <c r="Z29" s="3">
         <v>0.13811859200861359</v>
       </c>
-      <c r="AA29" s="2">
+      <c r="AA29" s="3">
         <v>0.1566567055638326</v>
       </c>
-      <c r="AB29" s="2">
+      <c r="AB29" s="3">
         <v>-7.7705292109581325E-2</v>
       </c>
-      <c r="AC29" s="2">
+      <c r="AC29" s="3">
         <v>0.10817931502983601</v>
       </c>
-      <c r="AD29" s="2">
+      <c r="AD29" s="3">
         <v>5.377222737175158E-2</v>
       </c>
-      <c r="AE29" s="2">
+      <c r="AE29" s="3">
         <v>0.1645435923658487</v>
       </c>
-      <c r="AF29" s="2">
+      <c r="AF29" s="3">
         <v>-5.5537819245731417E-2</v>
-      </c>
-      <c r="AG29">
-        <v>500438.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
765148 Adding a mandate to the IPS Generator (GMO US Equity)
</commit_message>
<xml_diff>
--- a/app/static/returns/returns.xlsx
+++ b/app/static/returns/returns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneaviso-my.sharepoint.com/personal/oelassaad_aviso_ca/Documents/Development/MAP Dev/performance-scripts/performance/IPS Quarterly Returns/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ips-generator-web\app\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{D7C4D0B6-8C0E-4FBE-B88D-53CF4D9F809E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72362337-A7B9-4B15-8A8F-441443B1DF44}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C791A5-5EAE-44F1-AF37-36C2F6658260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="83">
   <si>
     <t>Benchmark</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>2018a</t>
+  </si>
+  <si>
+    <t>GMO US Equity</t>
   </si>
 </sst>
 </file>
@@ -359,7 +362,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -370,6 +373,12 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -675,14 +684,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AG31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="95.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="95.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>74</v>
       </c>
@@ -781,7 +790,7 @@
       </c>
       <c r="AG1" s="1"/>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -882,7 +891,7 @@
         <v>39803186.619999997</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -983,7 +992,7 @@
         <v>94798917.329999998</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -1084,7 +1093,7 @@
         <v>222583420.25</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -1185,7 +1194,7 @@
         <v>23540552.809999999</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -1286,7 +1295,7 @@
         <v>33780758.009999998</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>29</v>
       </c>
@@ -1387,7 +1396,7 @@
         <v>90920741.019999996</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -1488,7 +1497,7 @@
         <v>147366568.47</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>31</v>
       </c>
@@ -1589,7 +1598,7 @@
         <v>46353484.43</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -1690,7 +1699,7 @@
         <v>24443101.23</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>33</v>
       </c>
@@ -1791,7 +1800,7 @@
         <v>107686266.65000001</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1892,7 +1901,7 @@
         <v>37634913.840000004</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>35</v>
       </c>
@@ -1993,7 +2002,7 @@
         <v>64605555.920000002</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>36</v>
       </c>
@@ -2094,7 +2103,7 @@
         <v>124488080.95999999</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -2195,7 +2204,7 @@
         <v>18199081.34</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
@@ -2296,7 +2305,7 @@
         <v>5692482.0300000003</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
@@ -2397,7 +2406,7 @@
         <v>27499642.469999999</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>40</v>
       </c>
@@ -2498,7 +2507,7 @@
         <v>25394222.760000002</v>
       </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>41</v>
       </c>
@@ -2599,7 +2608,7 @@
         <v>1392183.03</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>42</v>
       </c>
@@ -2700,7 +2709,7 @@
         <v>14695241.279999999</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>43</v>
       </c>
@@ -2801,7 +2810,7 @@
         <v>14813797.34</v>
       </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>44</v>
       </c>
@@ -2902,7 +2911,7 @@
         <v>21394718.059999999</v>
       </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>45</v>
       </c>
@@ -3003,7 +3012,7 @@
         <v>54504313.780000001</v>
       </c>
     </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
@@ -3104,7 +3113,7 @@
         <v>56551104.390000001</v>
       </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
@@ -3205,7 +3214,7 @@
         <v>179737885.86000001</v>
       </c>
     </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -3306,7 +3315,7 @@
         <v>2298181.69</v>
       </c>
     </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>49</v>
       </c>
@@ -3407,7 +3416,7 @@
         <v>13646549.710000001</v>
       </c>
     </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>272069.56</v>
       </c>
     </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>51</v>
       </c>
@@ -3609,7 +3618,7 @@
         <v>1652021.42</v>
       </c>
     </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>72</v>
       </c>
@@ -3705,10 +3714,109 @@
       </c>
       <c r="AF30">
         <v>1.0566379000000001E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="6">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="D31" s="6">
+        <v>5.04E-2</v>
+      </c>
+      <c r="E31" s="6">
+        <v>0.1231</v>
+      </c>
+      <c r="F31" s="6">
+        <v>9.8400000000000001E-2</v>
+      </c>
+      <c r="G31" s="6">
+        <v>0.2387</v>
+      </c>
+      <c r="H31" s="6">
+        <v>0.15890000000000001</v>
+      </c>
+      <c r="I31" s="6">
+        <v>0.1585</v>
+      </c>
+      <c r="J31" s="6">
+        <v>0.1048</v>
+      </c>
+      <c r="K31" s="7">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="L31" s="7">
+        <v>8.1199999999999994E-2</v>
+      </c>
+      <c r="M31" s="7">
+        <v>0.14829999999999999</v>
+      </c>
+      <c r="N31" s="7">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="O31" s="7">
+        <v>0.24929999999999999</v>
+      </c>
+      <c r="P31" s="7">
+        <v>0.16470000000000001</v>
+      </c>
+      <c r="Q31" s="7">
+        <v>0.153</v>
+      </c>
+      <c r="R31" s="7">
+        <v>0.10630000000000001</v>
+      </c>
+      <c r="S31" s="7">
+        <v>0.18859999999999999</v>
+      </c>
+      <c r="T31" s="7">
+        <v>0.29759999999999998</v>
+      </c>
+      <c r="U31" s="7">
+        <v>-0.15459999999999999</v>
+      </c>
+      <c r="V31" s="7">
+        <v>0.25850000000000001</v>
+      </c>
+      <c r="W31" s="7">
+        <v>0.1852</v>
+      </c>
+      <c r="X31" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="7">
+        <v>0.25019999999999998</v>
+      </c>
+      <c r="AA31" s="7">
+        <v>0.26290000000000002</v>
+      </c>
+      <c r="AB31" s="7">
+        <v>-0.18110000000000001</v>
+      </c>
+      <c r="AC31" s="7">
+        <v>0.28710000000000002</v>
+      </c>
+      <c r="AD31" s="7">
+        <v>0.184</v>
+      </c>
+      <c r="AE31">
+        <v>0</v>
+      </c>
+      <c r="AF31">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AG30" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat[pdf]: 142099 GMO US Equity changes and Fact sheets
</commit_message>
<xml_diff>
--- a/app/static/returns/returns.xlsx
+++ b/app/static/returns/returns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ips-generator-web\app\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C791A5-5EAE-44F1-AF37-36C2F6658260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EE543A-0CBE-44AE-B5F0-69333EF056FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -291,7 +291,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +313,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -362,7 +368,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -373,12 +379,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2312,95 +2313,95 @@
       <c r="B17" t="s">
         <v>64</v>
       </c>
-      <c r="C17">
-        <v>3.0806499999999959E-2</v>
-      </c>
-      <c r="D17">
-        <v>6.8728471042260209E-2</v>
-      </c>
-      <c r="E17">
-        <v>8.8490805068078826E-2</v>
-      </c>
-      <c r="F17">
-        <v>0.11876950311548209</v>
-      </c>
-      <c r="G17">
-        <v>0.1711255433792496</v>
-      </c>
-      <c r="H17">
-        <v>0.1050583256532238</v>
-      </c>
-      <c r="I17">
-        <v>0.1094534532033444</v>
-      </c>
-      <c r="J17">
-        <v>8.3498907775782616E-2</v>
-      </c>
-      <c r="K17">
-        <v>5.0200000000000022E-2</v>
-      </c>
-      <c r="L17">
-        <v>9.7537975039999836E-2</v>
-      </c>
-      <c r="M17">
-        <v>0.14596943571073909</v>
-      </c>
-      <c r="N17">
-        <v>0.2079818409207477</v>
-      </c>
-      <c r="O17">
-        <v>0.2370344962480708</v>
-      </c>
-      <c r="P17">
-        <v>0.14509477896558559</v>
-      </c>
-      <c r="Q17">
-        <v>0.1214983822931637</v>
-      </c>
-      <c r="R17">
-        <v>8.5472751656969992E-2</v>
-      </c>
-      <c r="S17">
-        <v>0.19251440061512121</v>
-      </c>
-      <c r="T17">
-        <v>0.14144707145853319</v>
-      </c>
-      <c r="U17">
-        <v>-0.119339609569489</v>
-      </c>
-      <c r="V17">
-        <v>0.17776070452224821</v>
-      </c>
-      <c r="W17">
-        <v>0.15429357627026061</v>
-      </c>
-      <c r="X17">
-        <v>0.19951799007801679</v>
-      </c>
-      <c r="Y17">
-        <v>1.175024958400717E-2</v>
-      </c>
-      <c r="Z17">
-        <v>0.2815483740958018</v>
-      </c>
-      <c r="AA17">
-        <v>0.19088023426714379</v>
-      </c>
-      <c r="AB17">
-        <v>-0.1242951408520198</v>
-      </c>
-      <c r="AC17">
-        <v>0.17523622407634301</v>
-      </c>
-      <c r="AD17">
-        <v>0.1225417737020502</v>
-      </c>
-      <c r="AE17">
-        <v>0.2019868939492451</v>
-      </c>
-      <c r="AF17">
-        <v>-1.2569244036318761E-2</v>
+      <c r="C17" s="6">
+        <v>3.0806500000000001E-2</v>
+      </c>
+      <c r="D17" s="6">
+        <v>6.8728470999999999E-2</v>
+      </c>
+      <c r="E17" s="6">
+        <v>4.1928640000000003E-2</v>
+      </c>
+      <c r="F17" s="6">
+        <v>7.0912111999999999E-2</v>
+      </c>
+      <c r="G17" s="6">
+        <v>0.154182603</v>
+      </c>
+      <c r="H17" s="6">
+        <v>9.5438102999999996E-2</v>
+      </c>
+      <c r="I17" s="6">
+        <v>0.104613655</v>
+      </c>
+      <c r="J17" s="6">
+        <v>8.1418746E-2</v>
+      </c>
+      <c r="K17" s="6">
+        <v>5.0200000000000002E-2</v>
+      </c>
+      <c r="L17" s="6">
+        <v>9.7537974999999999E-2</v>
+      </c>
+      <c r="M17" s="6">
+        <v>0.14596943600000001</v>
+      </c>
+      <c r="N17" s="6">
+        <v>0.207981841</v>
+      </c>
+      <c r="O17" s="6">
+        <v>0.23703449600000001</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0.14509477900000001</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>0.121498382</v>
+      </c>
+      <c r="R17" s="6">
+        <v>8.5472751999999999E-2</v>
+      </c>
+      <c r="S17" s="6">
+        <v>0.192514401</v>
+      </c>
+      <c r="T17" s="6">
+        <v>0.14144707100000001</v>
+      </c>
+      <c r="U17" s="6">
+        <v>-0.11933961</v>
+      </c>
+      <c r="V17" s="6">
+        <v>0.17776070499999999</v>
+      </c>
+      <c r="W17" s="6">
+        <v>0.15429357599999999</v>
+      </c>
+      <c r="X17" s="6">
+        <v>0.19951799000000001</v>
+      </c>
+      <c r="Y17" s="6">
+        <v>1.175025E-2</v>
+      </c>
+      <c r="Z17" s="6">
+        <v>0.28154837399999999</v>
+      </c>
+      <c r="AA17" s="6">
+        <v>0.19088023400000001</v>
+      </c>
+      <c r="AB17" s="6">
+        <v>-0.124295141</v>
+      </c>
+      <c r="AC17" s="6">
+        <v>0.175236224</v>
+      </c>
+      <c r="AD17" s="6">
+        <v>0.12254177400000001</v>
+      </c>
+      <c r="AE17" s="6">
+        <v>0.201986894</v>
+      </c>
+      <c r="AF17" s="6">
+        <v>-1.2569244E-2</v>
       </c>
       <c r="AG17">
         <v>27499642.469999999</v>
@@ -3723,95 +3724,95 @@
       <c r="B31" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="6">
-        <v>3.1600000000000003E-2</v>
-      </c>
-      <c r="D31" s="6">
+      <c r="C31" s="3">
+        <v>5.2671349581665972E-2</v>
+      </c>
+      <c r="D31" s="3">
+        <v>8.6286282420396265E-2</v>
+      </c>
+      <c r="E31" s="3">
+        <v>0.10502494093883263</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0.15862360534248277</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.26551179204480446</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0.20164784239868627</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0.18577241293856361</v>
+      </c>
+      <c r="J31" s="3">
+        <v>0.12082245611771181</v>
+      </c>
+      <c r="K31" s="3">
         <v>5.04E-2</v>
       </c>
-      <c r="E31" s="6">
-        <v>0.1231</v>
-      </c>
-      <c r="F31" s="6">
-        <v>9.8400000000000001E-2</v>
-      </c>
-      <c r="G31" s="6">
-        <v>0.2387</v>
-      </c>
-      <c r="H31" s="6">
-        <v>0.15890000000000001</v>
-      </c>
-      <c r="I31" s="6">
-        <v>0.1585</v>
-      </c>
-      <c r="J31" s="6">
-        <v>0.1048</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3.6499999999999998E-2</v>
-      </c>
-      <c r="L31" s="7">
-        <v>8.1199999999999994E-2</v>
-      </c>
-      <c r="M31" s="7">
-        <v>0.14829999999999999</v>
-      </c>
-      <c r="N31" s="7">
-        <v>0.17599999999999999</v>
-      </c>
-      <c r="O31" s="7">
-        <v>0.24929999999999999</v>
-      </c>
-      <c r="P31" s="7">
-        <v>0.16470000000000001</v>
-      </c>
-      <c r="Q31" s="7">
-        <v>0.153</v>
-      </c>
-      <c r="R31" s="7">
-        <v>0.10630000000000001</v>
-      </c>
-      <c r="S31" s="7">
-        <v>0.18859999999999999</v>
-      </c>
-      <c r="T31" s="7">
-        <v>0.29759999999999998</v>
-      </c>
-      <c r="U31" s="7">
-        <v>-0.15459999999999999</v>
-      </c>
-      <c r="V31" s="7">
-        <v>0.25850000000000001</v>
-      </c>
-      <c r="W31" s="7">
-        <v>0.1852</v>
-      </c>
-      <c r="X31" s="4">
-        <v>0</v>
-      </c>
-      <c r="Y31" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z31" s="7">
-        <v>0.25019999999999998</v>
-      </c>
-      <c r="AA31" s="7">
-        <v>0.26290000000000002</v>
-      </c>
-      <c r="AB31" s="7">
-        <v>-0.18110000000000001</v>
-      </c>
-      <c r="AC31" s="7">
-        <v>0.28710000000000002</v>
-      </c>
-      <c r="AD31" s="7">
-        <v>0.184</v>
-      </c>
-      <c r="AE31">
-        <v>0</v>
-      </c>
-      <c r="AF31">
-        <v>0</v>
+      <c r="L31" s="3">
+        <v>0.10257883008000013</v>
+      </c>
+      <c r="M31" s="3">
+        <v>0.11096858820849476</v>
+      </c>
+      <c r="N31" s="3">
+        <v>0.21124714771057596</v>
+      </c>
+      <c r="O31" s="3">
+        <v>0.25433471451881284</v>
+      </c>
+      <c r="P31" s="3">
+        <v>0.17409742870541312</v>
+      </c>
+      <c r="Q31" s="3">
+        <v>0.15675878094900253</v>
+      </c>
+      <c r="R31" s="3">
+        <v>0.10776062818835297</v>
+      </c>
+      <c r="S31" s="3">
+        <v>0.32019225783740701</v>
+      </c>
+      <c r="T31" s="3">
+        <v>0.3043959368722271</v>
+      </c>
+      <c r="U31" s="3">
+        <v>-8.859203546089589E-2</v>
+      </c>
+      <c r="V31" s="3">
+        <v>0.31520875441928764</v>
+      </c>
+      <c r="W31" s="3">
+        <v>0.15743636455567644</v>
+      </c>
+      <c r="X31" s="3">
+        <v>0.26804797435495398</v>
+      </c>
+      <c r="Y31" s="3">
+        <v>0.10909082769155654</v>
+      </c>
+      <c r="Z31" s="3">
+        <v>0.36378001862312792</v>
+      </c>
+      <c r="AA31" s="3">
+        <v>0.22802772224653478</v>
+      </c>
+      <c r="AB31" s="3">
+        <v>-0.12152410109852996</v>
+      </c>
+      <c r="AC31" s="3">
+        <v>0.2761454551589928</v>
+      </c>
+      <c r="AD31" s="3">
+        <v>0.15829193424188981</v>
+      </c>
+      <c r="AE31" s="3">
+        <v>0.24838940926861031</v>
+      </c>
+      <c r="AF31" s="3">
+        <v>4.2275010225730325E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update[perf]: 149272 updated q4 performance factsheets and minimum performance
</commit_message>
<xml_diff>
--- a/app/static/returns/returns.xlsx
+++ b/app/static/returns/returns.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneaviso-my.sharepoint.com/personal/oelassaad_aviso_ca/Documents/Development/MAP Dev/IPS Gen/ips-generator-web/app/static/returns/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ipsgenerator\ips-generator-web\app\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{D3EE543A-0CBE-44AE-B5F0-69333EF056FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECAF2DDA-865D-4C9B-8628-CC34070509E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8141C7BF-3282-4742-B4E7-39410A770314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>2019b</t>
   </si>
   <si>
-    <t>2018b</t>
-  </si>
-  <si>
     <t>Beutel Goodman Conservative Balanced</t>
   </si>
   <si>
@@ -272,9 +269,6 @@
     <t>2019a</t>
   </si>
   <si>
-    <t>2018a</t>
-  </si>
-  <si>
     <t>GMO US Equity</t>
   </si>
   <si>
@@ -282,6 +276,12 @@
   </si>
   <si>
     <t>Hamilton Lane Global Private Assets Fund</t>
+  </si>
+  <si>
+    <t>2025a</t>
+  </si>
+  <si>
+    <t>2025b</t>
   </si>
 </sst>
 </file>
@@ -351,15 +351,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,110 +675,110 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="Y1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="X1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="AG1" s="1"/>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
+      <c r="A2" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C2">
         <v>-1.035747368421047E-3</v>
@@ -872,11 +875,11 @@
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>25</v>
+      <c r="A3" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>-3.394180000000024E-3</v>
@@ -973,11 +976,11 @@
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>26</v>
+      <c r="A4" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4">
         <v>6.1357220338982277E-3</v>
@@ -1074,11 +1077,11 @@
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>27</v>
+      <c r="A5" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>2.3894181818182592E-3</v>
@@ -1175,11 +1178,11 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>28</v>
+      <c r="A6" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>8.3607619047618709E-3</v>
@@ -1276,11 +1279,11 @@
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>29</v>
+      <c r="A7" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>-7.6334545454544989E-3</v>
@@ -1377,11 +1380,11 @@
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>30</v>
+      <c r="A8" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>-2.477640571428574E-2</v>
@@ -1478,11 +1481,11 @@
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>31</v>
+      <c r="A9" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9">
         <v>-2.6760541666666641E-2</v>
@@ -1579,11 +1582,11 @@
       </c>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>32</v>
+      <c r="A10" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10">
         <v>9.0606296296296129E-3</v>
@@ -1680,11 +1683,11 @@
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>33</v>
+      <c r="A11" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11">
         <v>-1.081853688524592E-2</v>
@@ -1781,11 +1784,11 @@
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>34</v>
+      <c r="A12" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12">
         <v>-1.742916417910445E-2</v>
@@ -1882,11 +1885,11 @@
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>35</v>
+      <c r="A13" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13">
         <v>-5.137116666666719E-3</v>
@@ -1983,11 +1986,11 @@
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>36</v>
+      <c r="A14" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14">
         <v>1.169724161073815E-2</v>
@@ -2084,11 +2087,11 @@
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>37</v>
+      <c r="A15" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C15">
         <v>3.7355124999999927E-2</v>
@@ -2185,11 +2188,11 @@
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>38</v>
+      <c r="A16" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C16">
         <v>2.1268199999999959E-2</v>
@@ -2286,11 +2289,11 @@
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>39</v>
+      <c r="A17" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17">
         <v>-1.1736999999999999E-2</v>
@@ -2387,11 +2390,11 @@
       </c>
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>40</v>
+      <c r="A18" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C18">
         <v>6.3555277777778141E-3</v>
@@ -2488,11 +2491,11 @@
       </c>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>41</v>
+      <c r="A19" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19">
         <v>1.7811000000000021E-2</v>
@@ -2589,11 +2592,11 @@
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>42</v>
+      <c r="A20" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C20">
         <v>1.7353500000000022E-2</v>
@@ -2690,11 +2693,11 @@
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>43</v>
+      <c r="A21" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C21">
         <v>-1.225229999999999E-2</v>
@@ -2791,11 +2794,11 @@
       </c>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>44</v>
+      <c r="A22" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C22">
         <v>-8.9329999999999687E-3</v>
@@ -2892,11 +2895,11 @@
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>45</v>
+      <c r="A23" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>-2.2817100000000031E-2</v>
@@ -2993,11 +2996,11 @@
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>46</v>
+      <c r="A24" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C24">
         <v>2.3686040874457688E-3</v>
@@ -3094,11 +3097,11 @@
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>47</v>
+      <c r="A25" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C25">
         <v>2.2565704898560579E-3</v>
@@ -3195,11 +3198,11 @@
       </c>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>81</v>
+      <c r="A26" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26">
         <v>-8.80000000000003E-3</v>
@@ -3296,11 +3299,11 @@
       </c>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>48</v>
+      <c r="A27" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C27">
         <v>-2.3170000000000131E-3</v>
@@ -3397,11 +3400,11 @@
       </c>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>49</v>
+      <c r="A28" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28">
         <v>6.960999999999995E-3</v>
@@ -3498,11 +3501,11 @@
       </c>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" t="s">
         <v>69</v>
-      </c>
-      <c r="B29" t="s">
-        <v>70</v>
       </c>
       <c r="C29">
         <v>-4.9000000000000146E-3</v>
@@ -3517,13 +3520,13 @@
         <v>6.2204315008093307E-2</v>
       </c>
       <c r="G29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J29">
         <v>7.11764908177277E-2</v>
@@ -3541,13 +3544,13 @@
         <v>2.1108432930572851E-2</v>
       </c>
       <c r="O29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="P29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="R29">
         <v>4.7432916329392949E-2</v>
@@ -3559,19 +3562,19 @@
         <v>3.9763615369250223E-2</v>
       </c>
       <c r="U29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="V29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="W29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="X29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Y29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Z29">
         <v>2.1108432930572851E-2</v>
@@ -3580,30 +3583,30 @@
         <v>2.412349379091094E-2</v>
       </c>
       <c r="AB29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AC29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AD29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AE29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AF29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AG29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>79</v>
+      <c r="A30" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C30">
         <v>4.6999999999999256E-3</v>

</xml_diff>